<commit_message>
feat(finance): reconciliation periods, receivables reminders, finance reports
- Bank reconciliation by period with discrepancy items and resolution
- Advertiser receivables with payment reminders (ReceivableReminderEvent)
- Finance reports page and CSV export (httpClient.getFile)
- SePay log reference index, payment complaint and processing fixes
- Renumber local migrations to V10/V11 after main's V9 (advertising booking)
- Dev profile: enable spring.flyway.out-of-order so late-merged migrations apply
- AGENTS.md Rule 20: timestamp-based migration naming to avoid version clashes
</commit_message>
<xml_diff>
--- a/project_tracking_group2.xlsx
+++ b/project_tracking_group2.xlsx
@@ -2058,12 +2058,12 @@
       </c>
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>Create Payment Transaction</t>
+          <t>Create Payment Order</t>
         </is>
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>Reader, Advertiser, Payment Gateway</t>
+          <t>Reader, Advertiser</t>
         </is>
       </c>
       <c r="D48" s="25" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E48" s="26" t="inlineStr">
         <is>
-          <t>A payment transaction is created for Premium content or advertising.</t>
+          <t>SV1 / SV3 create a 15-minute PENDING order and send the customer to the shared payment page; every order is paid from the LocalPress wallet, a shortfall creates a top-up QR.</t>
         </is>
       </c>
       <c r="F48" s="22" t="n"/>
@@ -2088,12 +2088,12 @@
       </c>
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>Verify Payment Result</t>
+          <t>Verify SePay Payment</t>
         </is>
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>Payment Gateway, Staff</t>
+          <t>Payment Gateway (SePay), Accountant</t>
         </is>
       </c>
       <c r="D49" s="25" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="E49" s="26" t="inlineStr">
         <is>
-          <t>Payment result, amount, currency, and transaction reference are verified.</t>
+          <t>The system checks the SePay API key, finds the order code in the transfer content and compares the amount; every receipt is logged with its raw payload.</t>
         </is>
       </c>
       <c r="F49" s="22" t="n"/>
@@ -2118,12 +2118,12 @@
       </c>
       <c r="B50" s="26" t="inlineStr">
         <is>
-          <t>Handle Payment Webhook</t>
+          <t>Handle Payment Webhook (Idempotent)</t>
         </is>
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>Payment Gateway</t>
+          <t>Payment Gateway (SePay), SV1 / SV3 Modules</t>
         </is>
       </c>
       <c r="D50" s="25" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="E50" s="26" t="inlineStr">
         <is>
-          <t>The system authenticates and processes gateway webhooks without duplication.</t>
+          <t>The system processes each SePay transfer exactly once (unique sepay_id), credits the wallet, auto-pays the linked order and publishes PaymentSuccessEvent.</t>
         </is>
       </c>
       <c r="F50" s="22" t="n"/>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>Reader, Advertiser, Payment Gateway</t>
+          <t>Reader, Advertiser, Payment Gateway (SePay)</t>
         </is>
       </c>
       <c r="D51" s="25" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E51" s="26" t="inlineStr">
         <is>
-          <t>User checks the latest verified payment status.</t>
+          <t>The payment page polls the order status and can ask the SePay API directly; rights are never granted from the browser.</t>
         </is>
       </c>
       <c r="F51" s="22" t="n"/>
@@ -2178,12 +2178,12 @@
       </c>
       <c r="B52" s="26" t="inlineStr">
         <is>
-          <t>Confirm Manual Bank Transfer</t>
+          <t>Handle Unrecorded Payment Complaint</t>
         </is>
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Reader, Advertiser, Accountant, Bank Statement</t>
         </is>
       </c>
       <c r="D52" s="25" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="E52" s="26" t="inlineStr">
         <is>
-          <t>Staff matches a bank transfer with an order or advertising contract.</t>
+          <t>Customer reports a transfer that was not recorded; Accountant matches the bank statement and records it to the order, credits the wallet, or rejects with a reason.</t>
         </is>
       </c>
       <c r="F52" s="22" t="n"/>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Accountant, Chief Accountant</t>
         </is>
       </c>
       <c r="D53" s="25" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="E53" s="26" t="inlineStr">
         <is>
-          <t>Staff views Premium income, advertising income, fees, and refunds.</t>
+          <t>Accountant views net revenue (gross minus refunds, top-ups excluded), a 14-day chart and the to-do list.</t>
         </is>
       </c>
       <c r="F53" s="22" t="n"/>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>Staff, Advertiser</t>
+          <t>Accountant</t>
         </is>
       </c>
       <c r="D54" s="25" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E54" s="26" t="inlineStr">
         <is>
-          <t>Staff tracks advertising debts, payment periods, and due dates.</t>
+          <t>Accountant tracks advertising debts per campaign: paid in full, in term, overdue with days overdue.</t>
         </is>
       </c>
       <c r="F54" s="22" t="n"/>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>Staff, Payment Gateway</t>
+          <t>Accountant, Chief Accountant, Bank Statement</t>
         </is>
       </c>
       <c r="D55" s="25" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="E55" s="26" t="inlineStr">
         <is>
-          <t>Staff resolves mismatches between gateway, order, and access records.</t>
+          <t>Accountant compares system totals with the bank statement, resolves each mismatch with a note; Chief Accountant closes the period.</t>
         </is>
       </c>
       <c r="F55" s="22" t="n"/>
@@ -2298,12 +2298,12 @@
       </c>
       <c r="B56" s="26" t="inlineStr">
         <is>
-          <t>Process Refund Request</t>
+          <t>Process Refund Request (Four-Eyes)</t>
         </is>
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>Staff, Payment Gateway</t>
+          <t>Accountant, Chief Accountant</t>
         </is>
       </c>
       <c r="D56" s="25" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="E56" s="26" t="inlineStr">
         <is>
-          <t>Staff checks, approves, submits, and monitors a refund request.</t>
+          <t>Accountant proposes a refund within the amount collected; a different Chief Accountant approves or rejects it.</t>
         </is>
       </c>
       <c r="F56" s="22" t="n"/>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>System, SV1 / SV3 Modules</t>
         </is>
       </c>
       <c r="D57" s="25" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="E57" s="26" t="inlineStr">
         <is>
-          <t>Staff adjusts reading rights or campaign benefits after a refund.</t>
+          <t>A completed refund records a REFUND entry and publishes RefundCompletedEvent; SV1 / SV3 revoke rights on a full refund.</t>
         </is>
       </c>
       <c r="F57" s="22" t="n"/>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Accountant</t>
         </is>
       </c>
       <c r="D58" s="25" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E58" s="26" t="inlineStr">
         <is>
-          <t>Staff generates receipts and simulated financial documents.</t>
+          <t>Accountant opens an order and prints or saves the invoice / payment document for paid orders.</t>
         </is>
       </c>
       <c r="F58" s="22" t="n"/>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Accountant</t>
         </is>
       </c>
       <c r="D59" s="25" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="E59" s="26" t="inlineStr">
         <is>
-          <t>Staff views payment, fee, refund, and adjustment records.</t>
+          <t>Accountant views income and refund entries with net balance; wallet top-ups are a liability, not revenue.</t>
         </is>
       </c>
       <c r="F59" s="22" t="n"/>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Accountant, Chief Accountant</t>
         </is>
       </c>
       <c r="D60" s="25" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="E60" s="26" t="inlineStr">
         <is>
-          <t>Staff exports revenue, receivable, refund, and reconciliation reports.</t>
+          <t>Accountant exports transactions as CSV (UTF-8 with BOM for Excel).</t>
         </is>
       </c>
       <c r="F60" s="22" t="n"/>
@@ -2453,7 +2453,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>Staff, Notification Gateway</t>
+          <t>Accountant</t>
         </is>
       </c>
       <c r="D61" s="25" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="E61" s="26" t="inlineStr">
         <is>
-          <t>Staff views pending payments, webhook failures, and unresolved refunds.</t>
+          <t>Accountant views pending refunds, open complaints and overdue advertising debts, and opens the linked queue.</t>
         </is>
       </c>
       <c r="F61" s="22" t="n"/>
@@ -3898,7 +3898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AF53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" style="23" min="1" max="1"/>
@@ -3922,13 +3922,17 @@
     <col width="17" customWidth="1" style="23" min="19" max="19"/>
     <col width="15" customWidth="1" style="23" min="20" max="20"/>
     <col width="12" customWidth="1" style="23" min="21" max="21"/>
-    <col width="25" customWidth="1" style="23" min="22" max="22"/>
-    <col width="12" customWidth="1" style="23" min="23" max="23"/>
-    <col width="18" customWidth="1" style="23" min="24" max="24"/>
-    <col width="10" customWidth="1" style="23" min="25" max="25"/>
-    <col width="10" customWidth="1" style="23" min="26" max="26"/>
-    <col width="10" customWidth="1" style="23" min="27" max="27"/>
-    <col width="85" customWidth="1" style="23" min="28" max="28"/>
+    <col width="14" customWidth="1" style="23" min="22" max="22"/>
+    <col width="14" customWidth="1" style="23" min="23" max="23"/>
+    <col width="14" customWidth="1" style="23" min="24" max="24"/>
+    <col width="14" customWidth="1" style="23" min="25" max="25"/>
+    <col width="25" customWidth="1" style="23" min="26" max="26"/>
+    <col width="12" customWidth="1" style="23" min="27" max="27"/>
+    <col width="18" customWidth="1" style="23" min="28" max="28"/>
+    <col width="10" customWidth="1" style="23" min="29" max="29"/>
+    <col width="10" customWidth="1" style="23" min="30" max="30"/>
+    <col width="10" customWidth="1" style="23" min="31" max="31"/>
+    <col width="85" customWidth="1" style="23" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="23">
@@ -4039,35 +4043,55 @@
       </c>
       <c r="V1" s="24" t="inlineStr">
         <is>
+          <t>wallets</t>
+        </is>
+      </c>
+      <c r="W1" s="24" t="inlineStr">
+        <is>
+          <t>wallet_entries</t>
+        </is>
+      </c>
+      <c r="X1" s="24" t="inlineStr">
+        <is>
+          <t>sepay_webhook_logs</t>
+        </is>
+      </c>
+      <c r="Y1" s="24" t="inlineStr">
+        <is>
+          <t>payment_complaints</t>
+        </is>
+      </c>
+      <c r="Z1" s="24" t="inlineStr">
+        <is>
           <t>Use Cases</t>
         </is>
       </c>
-      <c r="W1" s="24" t="inlineStr">
+      <c r="AA1" s="24" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="X1" s="24" t="inlineStr">
+      <c r="AB1" s="24" t="inlineStr">
         <is>
           <t>In Charge</t>
         </is>
       </c>
-      <c r="Y1" s="24" t="inlineStr">
+      <c r="AC1" s="24" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="Z1" s="24" t="inlineStr">
+      <c r="AD1" s="24" t="inlineStr">
         <is>
           <t>SDS</t>
         </is>
       </c>
-      <c r="AA1" s="24" t="inlineStr">
+      <c r="AE1" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="AB1" s="24" t="inlineStr">
+      <c r="AF1" s="24" t="inlineStr">
         <is>
           <t>Notes / Updates</t>
         </is>
@@ -4111,37 +4135,41 @@
       <c r="S2" s="28" t="n"/>
       <c r="T2" s="28" t="n"/>
       <c r="U2" s="28" t="n"/>
-      <c r="V2" s="30" t="inlineStr">
+      <c r="V2" s="28" t="n"/>
+      <c r="W2" s="28" t="n"/>
+      <c r="X2" s="28" t="n"/>
+      <c r="Y2" s="28" t="n"/>
+      <c r="Z2" s="30" t="inlineStr">
         <is>
           <t>UC002</t>
         </is>
       </c>
-      <c r="W2" s="31" t="inlineStr">
+      <c r="AA2" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X2" s="28" t="inlineStr">
+      <c r="AB2" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y2" s="28" t="inlineStr">
+      <c r="AC2" s="28" t="inlineStr">
         <is>
           <t>II.1.1</t>
         </is>
       </c>
-      <c r="Z2" s="28" t="inlineStr">
+      <c r="AD2" s="28" t="inlineStr">
         <is>
           <t>II.1.1</t>
         </is>
       </c>
-      <c r="AA2" s="28" t="inlineStr">
+      <c r="AE2" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB2" s="30" t="inlineStr">
+      <c r="AF2" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Quản lý thông tin doanh nghiệp, mã số thuế, đại diện liên hệ, địa chỉ và hồ sơ năng lực.</t>
         </is>
@@ -4181,37 +4209,41 @@
       <c r="S3" s="28" t="n"/>
       <c r="T3" s="28" t="n"/>
       <c r="U3" s="28" t="n"/>
-      <c r="V3" s="30" t="inlineStr">
+      <c r="V3" s="28" t="n"/>
+      <c r="W3" s="28" t="n"/>
+      <c r="X3" s="28" t="n"/>
+      <c r="Y3" s="28" t="n"/>
+      <c r="Z3" s="30" t="inlineStr">
         <is>
           <t>UC003</t>
         </is>
       </c>
-      <c r="W3" s="31" t="inlineStr">
+      <c r="AA3" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X3" s="28" t="inlineStr">
+      <c r="AB3" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y3" s="28" t="inlineStr">
+      <c r="AC3" s="28" t="inlineStr">
         <is>
           <t>II.1.2</t>
         </is>
       </c>
-      <c r="Z3" s="28" t="inlineStr">
+      <c r="AD3" s="28" t="inlineStr">
         <is>
           <t>II.1.2</t>
         </is>
       </c>
-      <c r="AA3" s="28" t="inlineStr">
+      <c r="AE3" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB3" s="30" t="inlineStr">
+      <c r="AF3" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Tra cứu danh mục vị trí quảng cáo, kích thước banner, thiết bị hỗ trợ và bảng giá niêm yết.</t>
         </is>
@@ -4259,37 +4291,41 @@
       <c r="S4" s="28" t="n"/>
       <c r="T4" s="28" t="n"/>
       <c r="U4" s="28" t="n"/>
-      <c r="V4" s="30" t="inlineStr">
+      <c r="V4" s="28" t="n"/>
+      <c r="W4" s="28" t="n"/>
+      <c r="X4" s="28" t="n"/>
+      <c r="Y4" s="28" t="n"/>
+      <c r="Z4" s="30" t="inlineStr">
         <is>
           <t>UC004, UC005</t>
         </is>
       </c>
-      <c r="W4" s="32" t="inlineStr">
+      <c r="AA4" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X4" s="28" t="inlineStr">
+      <c r="AB4" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y4" s="28" t="inlineStr">
+      <c r="AC4" s="28" t="inlineStr">
         <is>
           <t>II.1.3</t>
         </is>
       </c>
-      <c r="Z4" s="28" t="inlineStr">
+      <c r="AD4" s="28" t="inlineStr">
         <is>
           <t>II.1.3</t>
         </is>
       </c>
-      <c r="AA4" s="28" t="inlineStr">
+      <c r="AE4" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB4" s="30" t="inlineStr">
+      <c r="AF4" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Chọn lịch chạy chiến dịch, kiểm tra chỗ trống (availability check), gửi yêu cầu booking slot.</t>
         </is>
@@ -4333,37 +4369,41 @@
       <c r="S5" s="28" t="n"/>
       <c r="T5" s="28" t="n"/>
       <c r="U5" s="28" t="n"/>
-      <c r="V5" s="30" t="inlineStr">
+      <c r="V5" s="28" t="n"/>
+      <c r="W5" s="28" t="n"/>
+      <c r="X5" s="28" t="n"/>
+      <c r="Y5" s="28" t="n"/>
+      <c r="Z5" s="30" t="inlineStr">
         <is>
           <t>UC006</t>
         </is>
       </c>
-      <c r="W5" s="32" t="inlineStr">
+      <c r="AA5" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X5" s="28" t="inlineStr">
+      <c r="AB5" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y5" s="28" t="inlineStr">
+      <c r="AC5" s="28" t="inlineStr">
         <is>
           <t>II.1.4</t>
         </is>
       </c>
-      <c r="Z5" s="28" t="inlineStr">
+      <c r="AD5" s="28" t="inlineStr">
         <is>
           <t>II.1.4</t>
         </is>
       </c>
-      <c r="AA5" s="28" t="inlineStr">
+      <c r="AE5" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB5" s="30" t="inlineStr">
+      <c r="AF5" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Xem bảng báo giá chính thức từ tòa soạn, xác nhận đơn giá, điều khoản hợp đồng trước khi trả tiền.</t>
         </is>
@@ -4411,37 +4451,41 @@
       <c r="S6" s="28" t="n"/>
       <c r="T6" s="28" t="n"/>
       <c r="U6" s="28" t="n"/>
-      <c r="V6" s="30" t="inlineStr">
+      <c r="V6" s="28" t="n"/>
+      <c r="W6" s="28" t="n"/>
+      <c r="X6" s="28" t="n"/>
+      <c r="Y6" s="28" t="n"/>
+      <c r="Z6" s="30" t="inlineStr">
         <is>
           <t>UC007</t>
         </is>
       </c>
-      <c r="W6" s="32" t="inlineStr">
+      <c r="AA6" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X6" s="28" t="inlineStr">
+      <c r="AB6" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y6" s="28" t="inlineStr">
+      <c r="AC6" s="28" t="inlineStr">
         <is>
           <t>II.1.5</t>
         </is>
       </c>
-      <c r="Z6" s="28" t="inlineStr">
+      <c r="AD6" s="28" t="inlineStr">
         <is>
           <t>II.1.5</t>
         </is>
       </c>
-      <c r="AA6" s="28" t="inlineStr">
+      <c r="AE6" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB6" s="30" t="inlineStr">
+      <c r="AF6" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Màn hình thanh toán đơn quảng cáo; kết nối module thanh toán SV4 để quét QR / nhận kết quả IPN.</t>
         </is>
@@ -4485,37 +4529,41 @@
       <c r="S7" s="28" t="n"/>
       <c r="T7" s="28" t="n"/>
       <c r="U7" s="28" t="n"/>
-      <c r="V7" s="30" t="inlineStr">
+      <c r="V7" s="28" t="n"/>
+      <c r="W7" s="28" t="n"/>
+      <c r="X7" s="28" t="n"/>
+      <c r="Y7" s="28" t="n"/>
+      <c r="Z7" s="30" t="inlineStr">
         <is>
           <t>UC008</t>
         </is>
       </c>
-      <c r="W7" s="32" t="inlineStr">
+      <c r="AA7" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X7" s="28" t="inlineStr">
+      <c r="AB7" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y7" s="28" t="inlineStr">
+      <c r="AC7" s="28" t="inlineStr">
         <is>
           <t>II.1.6</t>
         </is>
       </c>
-      <c r="Z7" s="28" t="inlineStr">
+      <c r="AD7" s="28" t="inlineStr">
         <is>
           <t>II.1.6</t>
         </is>
       </c>
-      <c r="AA7" s="28" t="inlineStr">
+      <c r="AE7" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB7" s="30" t="inlineStr">
+      <c r="AF7" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Upload banner quảng cáo, nhập URL đích, xem trước hiển thị thực tế (preview) theo slot tương ứng.</t>
         </is>
@@ -4575,37 +4623,41 @@
       <c r="S8" s="28" t="n"/>
       <c r="T8" s="28" t="n"/>
       <c r="U8" s="28" t="n"/>
-      <c r="V8" s="30" t="inlineStr">
+      <c r="V8" s="28" t="n"/>
+      <c r="W8" s="28" t="n"/>
+      <c r="X8" s="28" t="n"/>
+      <c r="Y8" s="28" t="n"/>
+      <c r="Z8" s="30" t="inlineStr">
         <is>
           <t>UC001, UC010, UC011</t>
         </is>
       </c>
-      <c r="W8" s="33" t="inlineStr">
+      <c r="AA8" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X8" s="28" t="inlineStr">
+      <c r="AB8" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y8" s="28" t="inlineStr">
+      <c r="AC8" s="28" t="inlineStr">
         <is>
           <t>II.1.7</t>
         </is>
       </c>
-      <c r="Z8" s="28" t="inlineStr">
+      <c r="AD8" s="28" t="inlineStr">
         <is>
           <t>II.1.7</t>
         </is>
       </c>
-      <c r="AA8" s="28" t="inlineStr">
+      <c r="AE8" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB8" s="30" t="inlineStr">
+      <c r="AF8" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Dashboard theo dõi chiến dịch đang chạy/hoàn tất, phân tích hiệu suất (Impressions, Clicks, CTR).</t>
         </is>
@@ -4649,37 +4701,41 @@
       <c r="S9" s="28" t="n"/>
       <c r="T9" s="28" t="n"/>
       <c r="U9" s="28" t="n"/>
-      <c r="V9" s="30" t="inlineStr">
+      <c r="V9" s="28" t="n"/>
+      <c r="W9" s="28" t="n"/>
+      <c r="X9" s="28" t="n"/>
+      <c r="Y9" s="28" t="n"/>
+      <c r="Z9" s="30" t="inlineStr">
         <is>
           <t>UC009</t>
         </is>
       </c>
-      <c r="W9" s="33" t="inlineStr">
+      <c r="AA9" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X9" s="28" t="inlineStr">
+      <c r="AB9" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y9" s="28" t="inlineStr">
+      <c r="AC9" s="28" t="inlineStr">
         <is>
           <t>II.1.8</t>
         </is>
       </c>
-      <c r="Z9" s="28" t="inlineStr">
+      <c r="AD9" s="28" t="inlineStr">
         <is>
           <t>II.1.8</t>
         </is>
       </c>
-      <c r="AA9" s="28" t="inlineStr">
+      <c r="AE9" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB9" s="30" t="inlineStr">
+      <c r="AF9" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Nộp banner mới hoặc đổi URL đích cho chiến dịch đang chạy; sinh creative version mới chờ duyệt.</t>
         </is>
@@ -4727,37 +4783,41 @@
         </is>
       </c>
       <c r="U10" s="28" t="n"/>
-      <c r="V10" s="30" t="inlineStr">
+      <c r="V10" s="28" t="n"/>
+      <c r="W10" s="28" t="n"/>
+      <c r="X10" s="28" t="n"/>
+      <c r="Y10" s="28" t="n"/>
+      <c r="Z10" s="30" t="inlineStr">
         <is>
           <t>UC013, UC014</t>
         </is>
       </c>
-      <c r="W10" s="33" t="inlineStr">
+      <c r="AA10" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X10" s="28" t="inlineStr">
+      <c r="AB10" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y10" s="28" t="inlineStr">
+      <c r="AC10" s="28" t="inlineStr">
         <is>
           <t>II.1.9</t>
         </is>
       </c>
-      <c r="Z10" s="28" t="inlineStr">
+      <c r="AD10" s="28" t="inlineStr">
         <is>
           <t>II.1.9</t>
         </is>
       </c>
-      <c r="AA10" s="28" t="inlineStr">
+      <c r="AE10" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB10" s="30" t="inlineStr">
+      <c r="AF10" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Gửi yêu cầu hủy booking / xin hoàn tiền; nhận thông báo trạng thái phê duyệt, lịch chạy, nhắc nợ.</t>
         </is>
@@ -4805,37 +4865,41 @@
       <c r="S11" s="28" t="n"/>
       <c r="T11" s="28" t="n"/>
       <c r="U11" s="28" t="n"/>
-      <c r="V11" s="30" t="inlineStr">
+      <c r="V11" s="28" t="n"/>
+      <c r="W11" s="28" t="n"/>
+      <c r="X11" s="28" t="n"/>
+      <c r="Y11" s="28" t="n"/>
+      <c r="Z11" s="30" t="inlineStr">
         <is>
           <t>UC012</t>
         </is>
       </c>
-      <c r="W11" s="33" t="inlineStr">
+      <c r="AA11" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X11" s="28" t="inlineStr">
+      <c r="AB11" s="28" t="inlineStr">
         <is>
           <t>SV1 (Tây)</t>
         </is>
       </c>
-      <c r="Y11" s="28" t="inlineStr">
+      <c r="AC11" s="28" t="inlineStr">
         <is>
           <t>II.1.10</t>
         </is>
       </c>
-      <c r="Z11" s="28" t="inlineStr">
+      <c r="AD11" s="28" t="inlineStr">
         <is>
           <t>II.1.10</t>
         </is>
       </c>
-      <c r="AA11" s="28" t="inlineStr">
+      <c r="AE11" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB11" s="30" t="inlineStr">
+      <c r="AF11" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Xem và tải về hợp đồng quảng cáo B2B, hóa đơn điện tử VAT, chứng từ thanh toán và biên bản nghiệm thu.</t>
         </is>
@@ -4883,37 +4947,41 @@
       <c r="S12" s="28" t="n"/>
       <c r="T12" s="28" t="n"/>
       <c r="U12" s="28" t="n"/>
-      <c r="V12" s="30" t="inlineStr">
+      <c r="V12" s="28" t="n"/>
+      <c r="W12" s="28" t="n"/>
+      <c r="X12" s="28" t="n"/>
+      <c r="Y12" s="28" t="n"/>
+      <c r="Z12" s="30" t="inlineStr">
         <is>
           <t>UC025</t>
         </is>
       </c>
-      <c r="W12" s="31" t="inlineStr">
+      <c r="AA12" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X12" s="28" t="inlineStr">
+      <c r="AB12" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y12" s="28" t="inlineStr">
+      <c r="AC12" s="28" t="inlineStr">
         <is>
           <t>II.2.1</t>
         </is>
       </c>
-      <c r="Z12" s="28" t="inlineStr">
+      <c r="AD12" s="28" t="inlineStr">
         <is>
           <t>II.2.1</t>
         </is>
       </c>
-      <c r="AA12" s="28" t="inlineStr">
+      <c r="AE12" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB12" s="30" t="inlineStr">
+      <c r="AF12" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Managing Editor kiểm duyệt bài viết nháp ban đầu, gửi phản hồi góp ý hoặc duyệt xuất bản.</t>
         </is>
@@ -4961,37 +5029,41 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V13" s="30" t="inlineStr">
+      <c r="V13" s="29" t="n"/>
+      <c r="W13" s="29" t="n"/>
+      <c r="X13" s="29" t="n"/>
+      <c r="Y13" s="29" t="n"/>
+      <c r="Z13" s="30" t="inlineStr">
         <is>
           <t>UC026, UC027, UC028</t>
         </is>
       </c>
-      <c r="W13" s="31" t="inlineStr">
+      <c r="AA13" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X13" s="28" t="inlineStr">
+      <c r="AB13" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y13" s="28" t="inlineStr">
+      <c r="AC13" s="28" t="inlineStr">
         <is>
           <t>II.2.2</t>
         </is>
       </c>
-      <c r="Z13" s="28" t="inlineStr">
+      <c r="AD13" s="28" t="inlineStr">
         <is>
           <t>II.2.2</t>
         </is>
       </c>
-      <c r="AA13" s="28" t="inlineStr">
+      <c r="AE13" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB13" s="30" t="inlineStr">
+      <c r="AF13" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Kiểm duyệt bình luận độc giả (PENDING -&gt; APPROVED/REJECTED), gỡ bỏ bình luận độc hại, vi phạm.</t>
         </is>
@@ -5039,37 +5111,41 @@
       <c r="S14" s="28" t="n"/>
       <c r="T14" s="28" t="n"/>
       <c r="U14" s="28" t="n"/>
-      <c r="V14" s="30" t="inlineStr">
+      <c r="V14" s="28" t="n"/>
+      <c r="W14" s="28" t="n"/>
+      <c r="X14" s="28" t="n"/>
+      <c r="Y14" s="28" t="n"/>
+      <c r="Z14" s="30" t="inlineStr">
         <is>
           <t>UC016</t>
         </is>
       </c>
-      <c r="W14" s="32" t="inlineStr">
+      <c r="AA14" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X14" s="28" t="inlineStr">
+      <c r="AB14" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y14" s="28" t="inlineStr">
+      <c r="AC14" s="28" t="inlineStr">
         <is>
           <t>II.2.3</t>
         </is>
       </c>
-      <c r="Z14" s="28" t="inlineStr">
+      <c r="AD14" s="28" t="inlineStr">
         <is>
           <t>II.2.3</t>
         </is>
       </c>
-      <c r="AA14" s="28" t="inlineStr">
+      <c r="AE14" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB14" s="30" t="inlineStr">
+      <c r="AF14" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Hàng đợi xử lý yêu cầu đặt quảng cáo của doanh nghiệp; nhân viên xem xét duyệt hoặc từ chối booking.</t>
         </is>
@@ -5113,37 +5189,41 @@
       <c r="S15" s="28" t="n"/>
       <c r="T15" s="28" t="n"/>
       <c r="U15" s="28" t="n"/>
-      <c r="V15" s="30" t="inlineStr">
+      <c r="V15" s="28" t="n"/>
+      <c r="W15" s="28" t="n"/>
+      <c r="X15" s="28" t="n"/>
+      <c r="Y15" s="28" t="n"/>
+      <c r="Z15" s="30" t="inlineStr">
         <is>
           <t>UC017</t>
         </is>
       </c>
-      <c r="W15" s="32" t="inlineStr">
+      <c r="AA15" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X15" s="28" t="inlineStr">
+      <c r="AB15" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y15" s="28" t="inlineStr">
+      <c r="AC15" s="28" t="inlineStr">
         <is>
           <t>II.2.4</t>
         </is>
       </c>
-      <c r="Z15" s="28" t="inlineStr">
+      <c r="AD15" s="28" t="inlineStr">
         <is>
           <t>II.2.4</t>
         </is>
       </c>
-      <c r="AA15" s="28" t="inlineStr">
+      <c r="AE15" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB15" s="30" t="inlineStr">
+      <c r="AF15" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Lịch trực quan quản lý sức chứa slot quảng cáo theo ngày/tuần/tháng; kiểm soát chống trùng lịch đặt.</t>
         </is>
@@ -5191,37 +5271,41 @@
       <c r="S16" s="28" t="n"/>
       <c r="T16" s="28" t="n"/>
       <c r="U16" s="28" t="n"/>
-      <c r="V16" s="30" t="inlineStr">
+      <c r="V16" s="28" t="n"/>
+      <c r="W16" s="28" t="n"/>
+      <c r="X16" s="28" t="n"/>
+      <c r="Y16" s="28" t="n"/>
+      <c r="Z16" s="30" t="inlineStr">
         <is>
           <t>UC018</t>
         </is>
       </c>
-      <c r="W16" s="32" t="inlineStr">
+      <c r="AA16" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X16" s="28" t="inlineStr">
+      <c r="AB16" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y16" s="28" t="inlineStr">
+      <c r="AC16" s="28" t="inlineStr">
         <is>
           <t>II.2.5</t>
         </is>
       </c>
-      <c r="Z16" s="28" t="inlineStr">
+      <c r="AD16" s="28" t="inlineStr">
         <is>
           <t>II.2.5</t>
         </is>
       </c>
-      <c r="AA16" s="28" t="inlineStr">
+      <c r="AE16" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB16" s="30" t="inlineStr">
+      <c r="AF16" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Soạn thảo, phê duyệt chính sách chiết khấu và gửi báo giá chính thức đến nhà quảng cáo.</t>
         </is>
@@ -5269,37 +5353,41 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V17" s="30" t="inlineStr">
+      <c r="V17" s="29" t="n"/>
+      <c r="W17" s="29" t="n"/>
+      <c r="X17" s="29" t="n"/>
+      <c r="Y17" s="29" t="n"/>
+      <c r="Z17" s="30" t="inlineStr">
         <is>
           <t>UC020, UC021, UC022</t>
         </is>
       </c>
-      <c r="W17" s="32" t="inlineStr">
+      <c r="AA17" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X17" s="28" t="inlineStr">
+      <c r="AB17" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y17" s="28" t="inlineStr">
+      <c r="AC17" s="28" t="inlineStr">
         <is>
           <t>II.2.6</t>
         </is>
       </c>
-      <c r="Z17" s="28" t="inlineStr">
+      <c r="AD17" s="28" t="inlineStr">
         <is>
           <t>II.2.6</t>
         </is>
       </c>
-      <c r="AA17" s="28" t="inlineStr">
+      <c r="AE17" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB17" s="30" t="inlineStr">
+      <c r="AF17" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Duyệt banner quảng cáo và URL đích; duyệt banner thay thế; gắn lý do từ chối nếu không đạt chuẩn.</t>
         </is>
@@ -5347,37 +5435,41 @@
       <c r="S18" s="28" t="n"/>
       <c r="T18" s="28" t="n"/>
       <c r="U18" s="28" t="n"/>
-      <c r="V18" s="30" t="inlineStr">
+      <c r="V18" s="28" t="n"/>
+      <c r="W18" s="28" t="n"/>
+      <c r="X18" s="28" t="n"/>
+      <c r="Y18" s="28" t="n"/>
+      <c r="Z18" s="30" t="inlineStr">
         <is>
           <t>UC023</t>
         </is>
       </c>
-      <c r="W18" s="33" t="inlineStr">
+      <c r="AA18" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X18" s="28" t="inlineStr">
+      <c r="AB18" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y18" s="28" t="inlineStr">
+      <c r="AC18" s="28" t="inlineStr">
         <is>
           <t>II.2.7</t>
         </is>
       </c>
-      <c r="Z18" s="28" t="inlineStr">
+      <c r="AD18" s="28" t="inlineStr">
         <is>
           <t>II.2.7</t>
         </is>
       </c>
-      <c r="AA18" s="28" t="inlineStr">
+      <c r="AE18" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB18" s="30" t="inlineStr">
+      <c r="AF18" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Kiểm tra tổng hợp điều kiện kích hoạt chiến dịch (đã thanh toán/hợp đồng hợp lệ, banner duyệt, slot trống).</t>
         </is>
@@ -5421,37 +5513,41 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V19" s="30" t="inlineStr">
+      <c r="V19" s="29" t="n"/>
+      <c r="W19" s="29" t="n"/>
+      <c r="X19" s="29" t="n"/>
+      <c r="Y19" s="29" t="n"/>
+      <c r="Z19" s="30" t="inlineStr">
         <is>
           <t>UC024</t>
         </is>
       </c>
-      <c r="W19" s="33" t="inlineStr">
+      <c r="AA19" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X19" s="28" t="inlineStr">
+      <c r="AB19" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y19" s="28" t="inlineStr">
+      <c r="AC19" s="28" t="inlineStr">
         <is>
           <t>II.2.8</t>
         </is>
       </c>
-      <c r="Z19" s="28" t="inlineStr">
+      <c r="AD19" s="28" t="inlineStr">
         <is>
           <t>II.2.8</t>
         </is>
       </c>
-      <c r="AA19" s="28" t="inlineStr">
+      <c r="AE19" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB19" s="30" t="inlineStr">
+      <c r="AF19" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Tạm dừng chiến dịch khẩn cấp (khi banner vi phạm/link chết) hoặc khôi phục chạy lại chiến dịch.</t>
         </is>
@@ -5499,37 +5595,41 @@
       <c r="S20" s="28" t="n"/>
       <c r="T20" s="28" t="n"/>
       <c r="U20" s="28" t="n"/>
-      <c r="V20" s="30" t="inlineStr">
+      <c r="V20" s="28" t="n"/>
+      <c r="W20" s="28" t="n"/>
+      <c r="X20" s="28" t="n"/>
+      <c r="Y20" s="28" t="n"/>
+      <c r="Z20" s="30" t="inlineStr">
         <is>
           <t>UC019</t>
         </is>
       </c>
-      <c r="W20" s="33" t="inlineStr">
+      <c r="AA20" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X20" s="28" t="inlineStr">
+      <c r="AB20" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y20" s="28" t="inlineStr">
+      <c r="AC20" s="28" t="inlineStr">
         <is>
           <t>II.2.9</t>
         </is>
       </c>
-      <c r="Z20" s="28" t="inlineStr">
+      <c r="AD20" s="28" t="inlineStr">
         <is>
           <t>II.2.9</t>
         </is>
       </c>
-      <c r="AA20" s="28" t="inlineStr">
+      <c r="AE20" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB20" s="30" t="inlineStr">
+      <c r="AF20" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Quản lý hợp đồng thương mại quảng cáo: số hợp đồng, ngày ký, giá trị cam kết, đính kèm file hợp đồng.</t>
         </is>
@@ -5585,37 +5685,41 @@
       <c r="S21" s="28" t="n"/>
       <c r="T21" s="28" t="n"/>
       <c r="U21" s="28" t="n"/>
-      <c r="V21" s="30" t="inlineStr">
+      <c r="V21" s="28" t="n"/>
+      <c r="W21" s="28" t="n"/>
+      <c r="X21" s="28" t="n"/>
+      <c r="Y21" s="28" t="n"/>
+      <c r="Z21" s="30" t="inlineStr">
         <is>
           <t>UC015</t>
         </is>
       </c>
-      <c r="W21" s="33" t="inlineStr">
+      <c r="AA21" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X21" s="28" t="inlineStr">
+      <c r="AB21" s="28" t="inlineStr">
         <is>
           <t>SV2 (Trọng Phan)</t>
         </is>
       </c>
-      <c r="Y21" s="28" t="inlineStr">
+      <c r="AC21" s="28" t="inlineStr">
         <is>
           <t>II.2.10</t>
         </is>
       </c>
-      <c r="Z21" s="28" t="inlineStr">
+      <c r="AD21" s="28" t="inlineStr">
         <is>
           <t>II.2.10</t>
         </is>
       </c>
-      <c r="AA21" s="28" t="inlineStr">
+      <c r="AE21" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB21" s="30" t="inlineStr">
+      <c r="AF21" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Dashboard điều hành tổng thể tòa soạn: tổng hợp hiệu suất, doanh thu quảng cáo và các vấn đề vận hành.</t>
         </is>
@@ -5667,37 +5771,41 @@
       <c r="S22" s="28" t="n"/>
       <c r="T22" s="28" t="n"/>
       <c r="U22" s="28" t="n"/>
-      <c r="V22" s="30" t="inlineStr">
+      <c r="V22" s="28" t="n"/>
+      <c r="W22" s="28" t="n"/>
+      <c r="X22" s="28" t="n"/>
+      <c r="Y22" s="28" t="n"/>
+      <c r="Z22" s="30" t="inlineStr">
         <is>
           <t>UC029, UC030</t>
         </is>
       </c>
-      <c r="W22" s="31" t="inlineStr">
+      <c r="AA22" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X22" s="28" t="inlineStr">
+      <c r="AB22" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y22" s="28" t="inlineStr">
+      <c r="AC22" s="28" t="inlineStr">
         <is>
           <t>II.3.1</t>
         </is>
       </c>
-      <c r="Z22" s="28" t="inlineStr">
+      <c r="AD22" s="28" t="inlineStr">
         <is>
           <t>II.3.1</t>
         </is>
       </c>
-      <c r="AA22" s="28" t="inlineStr">
+      <c r="AE22" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB22" s="30" t="inlineStr">
+      <c r="AF22" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Trang chủ báo điện tử, hiển thị tin mới, tin tiêu điểm theo chuyên mục; tìm kiếm bài viết Free.</t>
         </is>
@@ -5745,37 +5853,41 @@
       <c r="S23" s="28" t="n"/>
       <c r="T23" s="28" t="n"/>
       <c r="U23" s="28" t="n"/>
-      <c r="V23" s="30" t="inlineStr">
+      <c r="V23" s="28" t="n"/>
+      <c r="W23" s="28" t="n"/>
+      <c r="X23" s="28" t="n"/>
+      <c r="Y23" s="28" t="n"/>
+      <c r="Z23" s="30" t="inlineStr">
         <is>
           <t>UC031, UC032</t>
         </is>
       </c>
-      <c r="W23" s="31" t="inlineStr">
+      <c r="AA23" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X23" s="28" t="inlineStr">
+      <c r="AB23" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y23" s="28" t="inlineStr">
+      <c r="AC23" s="28" t="inlineStr">
         <is>
           <t>II.3.2</t>
         </is>
       </c>
-      <c r="Z23" s="28" t="inlineStr">
+      <c r="AD23" s="28" t="inlineStr">
         <is>
           <t>II.3.2</t>
         </is>
       </c>
-      <c r="AA23" s="28" t="inlineStr">
+      <c r="AE23" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB23" s="30" t="inlineStr">
+      <c r="AF23" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Trang chi tiết đọc bài Free toàn văn, tự động tăng view count, hiển thị danh sách bình luận đã duyệt.</t>
         </is>
@@ -5819,37 +5931,41 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V24" s="30" t="inlineStr">
+      <c r="V24" s="29" t="n"/>
+      <c r="W24" s="29" t="n"/>
+      <c r="X24" s="29" t="n"/>
+      <c r="Y24" s="29" t="n"/>
+      <c r="Z24" s="30" t="inlineStr">
         <is>
           <t>UC033</t>
         </is>
       </c>
-      <c r="W24" s="31" t="inlineStr">
+      <c r="AA24" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X24" s="28" t="inlineStr">
+      <c r="AB24" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y24" s="28" t="inlineStr">
+      <c r="AC24" s="28" t="inlineStr">
         <is>
           <t>II.3.3</t>
         </is>
       </c>
-      <c r="Z24" s="28" t="inlineStr">
+      <c r="AD24" s="28" t="inlineStr">
         <is>
           <t>II.3.3</t>
         </is>
       </c>
-      <c r="AA24" s="28" t="inlineStr">
+      <c r="AE24" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB24" s="30" t="inlineStr">
+      <c r="AF24" s="30" t="inlineStr">
         <is>
           <t>[Đầu quy trình] Đăng ký, đăng nhập tài khoản độc giả (BCrypt hash), quên mật khẩu, cập nhật thông tin cá nhân.</t>
         </is>
@@ -5901,37 +6017,41 @@
       <c r="S25" s="28" t="n"/>
       <c r="T25" s="28" t="n"/>
       <c r="U25" s="28" t="n"/>
-      <c r="V25" s="30" t="inlineStr">
+      <c r="V25" s="28" t="n"/>
+      <c r="W25" s="28" t="n"/>
+      <c r="X25" s="28" t="n"/>
+      <c r="Y25" s="28" t="n"/>
+      <c r="Z25" s="30" t="inlineStr">
         <is>
           <t>UC034, UC035</t>
         </is>
       </c>
-      <c r="W25" s="32" t="inlineStr">
+      <c r="AA25" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X25" s="28" t="inlineStr">
+      <c r="AB25" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y25" s="28" t="inlineStr">
+      <c r="AC25" s="28" t="inlineStr">
         <is>
           <t>II.3.4</t>
         </is>
       </c>
-      <c r="Z25" s="28" t="inlineStr">
+      <c r="AD25" s="28" t="inlineStr">
         <is>
           <t>II.3.4</t>
         </is>
       </c>
-      <c r="AA25" s="28" t="inlineStr">
+      <c r="AE25" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB25" s="30" t="inlineStr">
+      <c r="AF25" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Giao diện chọn gói thuê bao (tháng/năm) hoặc mua lẻ từng bài viết; chuyển tiếp tạo đơn sang SV4.</t>
         </is>
@@ -5983,37 +6103,41 @@
       <c r="S26" s="28" t="n"/>
       <c r="T26" s="28" t="n"/>
       <c r="U26" s="28" t="n"/>
-      <c r="V26" s="30" t="inlineStr">
+      <c r="V26" s="28" t="n"/>
+      <c r="W26" s="28" t="n"/>
+      <c r="X26" s="28" t="n"/>
+      <c r="Y26" s="28" t="n"/>
+      <c r="Z26" s="30" t="inlineStr">
         <is>
           <t>UC036</t>
         </is>
       </c>
-      <c r="W26" s="32" t="inlineStr">
+      <c r="AA26" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X26" s="28" t="inlineStr">
+      <c r="AB26" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y26" s="28" t="inlineStr">
+      <c r="AC26" s="28" t="inlineStr">
         <is>
           <t>II.3.5</t>
         </is>
       </c>
-      <c r="Z26" s="28" t="inlineStr">
+      <c r="AD26" s="28" t="inlineStr">
         <is>
           <t>II.3.5</t>
         </is>
       </c>
-      <c r="AA26" s="28" t="inlineStr">
+      <c r="AE26" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB26" s="30" t="inlineStr">
+      <c r="AF26" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Đọc bài Premium; gọi PaywallEngine kiểm tra quyền (nếu chưa mua chỉ trả preview 30% nội dung từ máy chủ).</t>
         </is>
@@ -6061,37 +6185,41 @@
       <c r="S27" s="28" t="n"/>
       <c r="T27" s="28" t="n"/>
       <c r="U27" s="28" t="n"/>
-      <c r="V27" s="30" t="inlineStr">
+      <c r="V27" s="28" t="n"/>
+      <c r="W27" s="28" t="n"/>
+      <c r="X27" s="28" t="n"/>
+      <c r="Y27" s="28" t="n"/>
+      <c r="Z27" s="30" t="inlineStr">
         <is>
           <t>UC037, UC038, UC039</t>
         </is>
       </c>
-      <c r="W27" s="32" t="inlineStr">
+      <c r="AA27" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X27" s="28" t="inlineStr">
+      <c r="AB27" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y27" s="28" t="inlineStr">
+      <c r="AC27" s="28" t="inlineStr">
         <is>
           <t>II.3.6</t>
         </is>
       </c>
-      <c r="Z27" s="28" t="inlineStr">
+      <c r="AD27" s="28" t="inlineStr">
         <is>
           <t>II.3.6</t>
         </is>
       </c>
-      <c r="AA27" s="28" t="inlineStr">
+      <c r="AE27" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB27" s="30" t="inlineStr">
+      <c r="AF27" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Tủ sách cá nhân của độc giả: Quản lý bài đã lưu (bookmark), xem lịch sử đọc báo, danh sách bài lẻ đã mua.</t>
         </is>
@@ -6139,37 +6267,41 @@
       <c r="S28" s="28" t="n"/>
       <c r="T28" s="28" t="n"/>
       <c r="U28" s="28" t="n"/>
-      <c r="V28" s="30" t="inlineStr">
+      <c r="V28" s="28" t="n"/>
+      <c r="W28" s="28" t="n"/>
+      <c r="X28" s="28" t="n"/>
+      <c r="Y28" s="28" t="n"/>
+      <c r="Z28" s="30" t="inlineStr">
         <is>
           <t>UC041, UC042</t>
         </is>
       </c>
-      <c r="W28" s="32" t="inlineStr">
+      <c r="AA28" s="32" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X28" s="28" t="inlineStr">
+      <c r="AB28" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y28" s="28" t="inlineStr">
+      <c r="AC28" s="28" t="inlineStr">
         <is>
           <t>II.3.7</t>
         </is>
       </c>
-      <c r="Z28" s="28" t="inlineStr">
+      <c r="AD28" s="28" t="inlineStr">
         <is>
           <t>II.3.7</t>
         </is>
       </c>
-      <c r="AA28" s="28" t="inlineStr">
+      <c r="AE28" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB28" s="30" t="inlineStr">
+      <c r="AF28" s="30" t="inlineStr">
         <is>
           <t>[Giữa quy trình] Gửi bình luận vào bài viết (chuyển trạng thái PENDING); báo cáo bình luận xấu/vi phạm quy chuẩn.</t>
         </is>
@@ -6217,37 +6349,41 @@
       <c r="S29" s="28" t="n"/>
       <c r="T29" s="28" t="n"/>
       <c r="U29" s="28" t="n"/>
-      <c r="V29" s="30" t="inlineStr">
+      <c r="V29" s="28" t="n"/>
+      <c r="W29" s="28" t="n"/>
+      <c r="X29" s="28" t="n"/>
+      <c r="Y29" s="28" t="n"/>
+      <c r="Z29" s="30" t="inlineStr">
         <is>
           <t>UC040</t>
         </is>
       </c>
-      <c r="W29" s="33" t="inlineStr">
+      <c r="AA29" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X29" s="28" t="inlineStr">
+      <c r="AB29" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y29" s="28" t="inlineStr">
+      <c r="AC29" s="28" t="inlineStr">
         <is>
           <t>II.3.8</t>
         </is>
       </c>
-      <c r="Z29" s="28" t="inlineStr">
+      <c r="AD29" s="28" t="inlineStr">
         <is>
           <t>II.3.8</t>
         </is>
       </c>
-      <c r="AA29" s="28" t="inlineStr">
+      <c r="AE29" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB29" s="30" t="inlineStr">
+      <c r="AF29" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Quản lý danh sách chuyên mục địa phương hoặc tác giả đang theo dõi; luồng feed bài viết cá nhân hóa.</t>
         </is>
@@ -6291,37 +6427,41 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V30" s="30" t="inlineStr">
+      <c r="V30" s="29" t="n"/>
+      <c r="W30" s="29" t="n"/>
+      <c r="X30" s="29" t="n"/>
+      <c r="Y30" s="29" t="n"/>
+      <c r="Z30" s="30" t="inlineStr">
         <is>
           <t>UC043</t>
         </is>
       </c>
-      <c r="W30" s="33" t="inlineStr">
+      <c r="AA30" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X30" s="28" t="inlineStr">
+      <c r="AB30" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y30" s="28" t="inlineStr">
+      <c r="AC30" s="28" t="inlineStr">
         <is>
           <t>II.3.9</t>
         </is>
       </c>
-      <c r="Z30" s="28" t="inlineStr">
+      <c r="AD30" s="28" t="inlineStr">
         <is>
           <t>II.3.9</t>
         </is>
       </c>
-      <c r="AA30" s="28" t="inlineStr">
+      <c r="AE30" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB30" s="30" t="inlineStr">
+      <c r="AF30" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Quản lý phiên đăng nhập và thiết bị của độc giả; hiển thị cảnh báo và đá phiên khi vượt hạn mức 2 thiết bị.</t>
         </is>
@@ -6369,37 +6509,41 @@
       </c>
       <c r="T31" s="28" t="n"/>
       <c r="U31" s="28" t="n"/>
-      <c r="V31" s="30" t="inlineStr">
+      <c r="V31" s="28" t="n"/>
+      <c r="W31" s="28" t="n"/>
+      <c r="X31" s="28" t="n"/>
+      <c r="Y31" s="28" t="n"/>
+      <c r="Z31" s="30" t="inlineStr">
         <is>
           <t>UC044, UC045, UC046</t>
         </is>
       </c>
-      <c r="W31" s="33" t="inlineStr">
+      <c r="AA31" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X31" s="28" t="inlineStr">
+      <c r="AB31" s="28" t="inlineStr">
         <is>
           <t>SV3 (Hoàng)</t>
         </is>
       </c>
-      <c r="Y31" s="28" t="inlineStr">
+      <c r="AC31" s="28" t="inlineStr">
         <is>
           <t>II.3.10</t>
         </is>
       </c>
-      <c r="Z31" s="28" t="inlineStr">
+      <c r="AD31" s="28" t="inlineStr">
         <is>
           <t>II.3.10</t>
         </is>
       </c>
-      <c r="AA31" s="28" t="inlineStr">
+      <c r="AE31" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB31" s="30" t="inlineStr">
+      <c r="AF31" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Lịch sử giao dịch mua gói/bài lẻ; cấu hình tự động gia hạn thuê bao; gửi yêu cầu khiếu nại và xin hoàn tiền.</t>
         </is>
@@ -6408,7 +6552,7 @@
     <row r="32" ht="24" customHeight="1" s="23">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>Financial Documents and Ledger</t>
+          <t>Payment Checkout</t>
         </is>
       </c>
       <c r="B32" s="28" t="inlineStr">
@@ -6416,11 +6560,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C32" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="C32" s="29" t="n"/>
       <c r="D32" s="28" t="n"/>
       <c r="E32" s="28" t="n"/>
       <c r="F32" s="28" t="n"/>
@@ -6430,63 +6570,71 @@
       <c r="J32" s="28" t="n"/>
       <c r="K32" s="28" t="n"/>
       <c r="L32" s="28" t="n"/>
-      <c r="M32" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="M32" s="29" t="n"/>
       <c r="N32" s="28" t="n"/>
       <c r="O32" s="28" t="n"/>
       <c r="P32" s="28" t="n"/>
       <c r="Q32" s="28" t="n"/>
       <c r="R32" s="29" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="S32" s="28" t="n"/>
       <c r="T32" s="28" t="n"/>
       <c r="U32" s="28" t="n"/>
-      <c r="V32" s="30" t="inlineStr">
-        <is>
-          <t>UC057, UC058</t>
-        </is>
-      </c>
-      <c r="W32" s="31" t="inlineStr">
+      <c r="V32" s="28" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="W32" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X32" s="28" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="30" t="inlineStr">
+        <is>
+          <t>UC047, UC050</t>
+        </is>
+      </c>
+      <c r="AA32" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X32" s="28" t="inlineStr">
+      <c r="AB32" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y32" s="28" t="inlineStr">
+      <c r="AC32" s="28" t="inlineStr">
         <is>
           <t>II.4.1</t>
         </is>
       </c>
-      <c r="Z32" s="28" t="inlineStr">
+      <c r="AD32" s="28" t="inlineStr">
         <is>
           <t>II.4.1</t>
         </is>
       </c>
-      <c r="AA32" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB32" s="30" t="inlineStr">
-        <is>
-          <t>[Đầu quy trình] Sổ cái ghi nhận dòng tiền giao dịch; phát hành và quản lý hóa đơn VAT điện tử, biên nhận thu tiền.</t>
+      <c r="AE32" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF32" s="30" t="inlineStr">
+        <is>
+          <t>[Đầu quy trình] Trang thanh toán chung, mọi đơn trả bằng ví: ví đủ -&gt; 1 nút trừ ví (khóa dòng đơn + ví, 402 thiếu tiền, 410 hết hạn); ví thiếu -&gt; QR nạp bù đúng phần thiếu (shortfall-topup, dùng lại mã còn hạn), tiền về tự trả đơn. Polling 3 giây, kiểm tra lại qua API SePay. Không phải chủ đơn -&gt; 403. Route: /payment/:orderCode</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1" s="23">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>Manual Bank Transfer Confirmation</t>
+          <t>LocalPress Wallet and Top-up</t>
         </is>
       </c>
       <c r="B33" s="28" t="inlineStr">
@@ -6494,7 +6642,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C33" s="28" t="n"/>
+      <c r="C33" s="29" t="n"/>
       <c r="D33" s="28" t="n"/>
       <c r="E33" s="28" t="n"/>
       <c r="F33" s="28" t="n"/>
@@ -6504,71 +6652,79 @@
       <c r="J33" s="28" t="n"/>
       <c r="K33" s="28" t="n"/>
       <c r="L33" s="28" t="n"/>
-      <c r="M33" s="28" t="n"/>
+      <c r="M33" s="29" t="n"/>
       <c r="N33" s="28" t="n"/>
       <c r="O33" s="28" t="n"/>
       <c r="P33" s="28" t="n"/>
       <c r="Q33" s="28" t="n"/>
       <c r="R33" s="29" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>C</t>
         </is>
       </c>
       <c r="S33" s="28" t="n"/>
       <c r="T33" s="28" t="n"/>
-      <c r="U33" s="29" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V33" s="30" t="inlineStr">
-        <is>
-          <t>UC051</t>
-        </is>
-      </c>
-      <c r="W33" s="31" t="inlineStr">
+      <c r="U33" s="28" t="n"/>
+      <c r="V33" s="28" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="W33" s="28" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="X33" s="28" t="n"/>
+      <c r="Y33" s="28" t="n"/>
+      <c r="Z33" s="30" t="inlineStr">
+        <is>
+          <t>UC047, UC050</t>
+        </is>
+      </c>
+      <c r="AA33" s="31" t="inlineStr">
         <is>
           <t>Iter 1</t>
         </is>
       </c>
-      <c r="X33" s="28" t="inlineStr">
+      <c r="AB33" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y33" s="28" t="inlineStr">
+      <c r="AC33" s="28" t="inlineStr">
         <is>
           <t>II.4.2</t>
         </is>
       </c>
-      <c r="Z33" s="28" t="inlineStr">
+      <c r="AD33" s="28" t="inlineStr">
         <is>
           <t>II.4.2</t>
         </is>
       </c>
-      <c r="AA33" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB33" s="30" t="inlineStr">
-        <is>
-          <t>[Đầu quy trình] Kế toán đối chiếu sao kê tài khoản ngân hàng và xác nhận duyệt đơn chuyển khoản thủ công.</t>
+      <c r="AE33" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF33" s="30" t="inlineStr">
+        <is>
+          <t>[Đầu quy trình] Số dư + lịch sử ví; nạp tiền 10.000 - 50.000.000 ₫ (bội số 1.000) tạo đơn TOPUP rồi sang trang thanh toán chung. Tiền nạp là công nợ phải trả khách, không phải doanh thu. Route: /wallet, /wallet/topup</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="23">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>Payment Processing</t>
+          <t>SePay Webhook and Payment Log</t>
         </is>
       </c>
       <c r="B34" s="28" t="inlineStr">
         <is>
-          <t>Screen</t>
-        </is>
-      </c>
-      <c r="C34" s="28" t="n"/>
+          <t>Screen + API</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="n"/>
       <c r="D34" s="28" t="n"/>
       <c r="E34" s="28" t="n"/>
       <c r="F34" s="28" t="n"/>
@@ -6576,73 +6732,77 @@
       <c r="H34" s="28" t="n"/>
       <c r="I34" s="28" t="n"/>
       <c r="J34" s="28" t="n"/>
-      <c r="K34" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="L34" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="M34" s="28" t="n"/>
+      <c r="K34" s="28" t="n"/>
+      <c r="L34" s="28" t="n"/>
+      <c r="M34" s="29" t="n"/>
       <c r="N34" s="28" t="n"/>
-      <c r="O34" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="O34" s="28" t="n"/>
       <c r="P34" s="28" t="n"/>
       <c r="Q34" s="28" t="n"/>
       <c r="R34" s="29" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="S34" s="28" t="n"/>
       <c r="T34" s="28" t="n"/>
       <c r="U34" s="28" t="n"/>
-      <c r="V34" s="30" t="inlineStr">
-        <is>
-          <t>UC047, UC048, UC049, UC050</t>
-        </is>
-      </c>
-      <c r="W34" s="32" t="inlineStr">
-        <is>
-          <t>Iter 2</t>
+      <c r="V34" s="28" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="W34" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="X34" s="28" t="inlineStr">
         <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="Y34" s="28" t="n"/>
+      <c r="Z34" s="30" t="inlineStr">
+        <is>
+          <t>UC048, UC049</t>
+        </is>
+      </c>
+      <c r="AA34" s="31" t="inlineStr">
+        <is>
+          <t>Iter 1</t>
+        </is>
+      </c>
+      <c r="AB34" s="28" t="inlineStr">
+        <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y34" s="28" t="inlineStr">
+      <c r="AC34" s="28" t="inlineStr">
         <is>
           <t>II.4.3</t>
         </is>
       </c>
-      <c r="Z34" s="28" t="inlineStr">
+      <c r="AD34" s="28" t="inlineStr">
         <is>
           <t>II.4.3</t>
         </is>
       </c>
-      <c r="AA34" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB34" s="30" t="inlineStr">
-        <is>
-          <t>[Giữa quy trình] Khởi tạo mã VietQR/cổng thanh toán (VNPay/MoMo); xử lý Webhook IPN idempotent, cập nhật giao dịch tự động.</t>
+      <c r="AE34" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF34" s="30" t="inlineStr">
+        <is>
+          <t>[Đầu quy trình] Webhook SePay (API Key, idempotent theo sepay_id) + nhật ký từng lần tiền về kèm payload gốc; đồng bộ dự phòng qua API SePay. Kế toán xem nguồn Webhook / Đồng bộ API / Giả lập. Cần tunnel để SePay gọi vào máy local. Route: /backoffice/finance/sepay</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" s="23">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>Advertiser Receivables</t>
+          <t>Payment Complaint (Customer)</t>
         </is>
       </c>
       <c r="B35" s="28" t="inlineStr">
@@ -6650,7 +6810,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C35" s="28" t="n"/>
+      <c r="C35" s="29" t="n"/>
       <c r="D35" s="28" t="n"/>
       <c r="E35" s="28" t="n"/>
       <c r="F35" s="28" t="n"/>
@@ -6660,17 +6820,9 @@
       <c r="J35" s="28" t="n"/>
       <c r="K35" s="28" t="n"/>
       <c r="L35" s="28" t="n"/>
-      <c r="M35" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="M35" s="29" t="n"/>
       <c r="N35" s="28" t="n"/>
-      <c r="O35" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="O35" s="28" t="n"/>
       <c r="P35" s="28" t="n"/>
       <c r="Q35" s="28" t="n"/>
       <c r="R35" s="29" t="inlineStr">
@@ -6681,39 +6833,47 @@
       <c r="S35" s="28" t="n"/>
       <c r="T35" s="28" t="n"/>
       <c r="U35" s="28" t="n"/>
-      <c r="V35" s="30" t="inlineStr">
-        <is>
-          <t>UC053</t>
-        </is>
-      </c>
-      <c r="W35" s="32" t="inlineStr">
+      <c r="V35" s="28" t="n"/>
+      <c r="W35" s="28" t="n"/>
+      <c r="X35" s="28" t="n"/>
+      <c r="Y35" s="28" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="Z35" s="30" t="inlineStr">
+        <is>
+          <t>UC051</t>
+        </is>
+      </c>
+      <c r="AA35" s="31" t="inlineStr">
         <is>
           <t>Iter 2</t>
         </is>
       </c>
-      <c r="X35" s="28" t="inlineStr">
+      <c r="AB35" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y35" s="28" t="inlineStr">
+      <c r="AC35" s="28" t="inlineStr">
         <is>
           <t>II.4.4</t>
         </is>
       </c>
-      <c r="Z35" s="28" t="inlineStr">
+      <c r="AD35" s="28" t="inlineStr">
         <is>
           <t>II.4.4</t>
         </is>
       </c>
-      <c r="AA35" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB35" s="30" t="inlineStr">
-        <is>
-          <t>[Giữa quy trình] Theo dõi công nợ khách hàng quảng cáo B2B, quản lý thời hạn tín dụng và kích hoạt gửi thông báo nhắc nợ.</t>
+      <c r="AE35" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF35" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Khách gửi khiếu nại đã chuyển tiền chưa được ghi nhận: số tiền, thời gian, mã GD ngân hàng (UNIQUE, 409 nếu trùng), mã đơn (404 nếu không có, 403 nếu của người khác); theo dõi phản hồi của kế toán. Route: /wallet/complaints</t>
         </is>
       </c>
     </row>
@@ -6728,7 +6888,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C36" s="28" t="n"/>
+      <c r="C36" s="29" t="n"/>
       <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
       <c r="F36" s="28" t="n"/>
@@ -6738,7 +6898,7 @@
       <c r="J36" s="28" t="n"/>
       <c r="K36" s="28" t="n"/>
       <c r="L36" s="28" t="n"/>
-      <c r="M36" s="28" t="n"/>
+      <c r="M36" s="29" t="n"/>
       <c r="N36" s="28" t="n"/>
       <c r="O36" s="28" t="n"/>
       <c r="P36" s="28" t="n"/>
@@ -6748,53 +6908,61 @@
           <t>R</t>
         </is>
       </c>
-      <c r="S36" s="29" t="inlineStr">
+      <c r="S36" s="28" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
       <c r="T36" s="28" t="n"/>
       <c r="U36" s="28" t="n"/>
-      <c r="V36" s="30" t="inlineStr">
+      <c r="V36" s="28" t="n"/>
+      <c r="W36" s="28" t="n"/>
+      <c r="X36" s="28" t="n"/>
+      <c r="Y36" s="28" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Z36" s="30" t="inlineStr">
         <is>
           <t>UC052</t>
         </is>
       </c>
-      <c r="W36" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X36" s="28" t="inlineStr">
+      <c r="AA36" s="31" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB36" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y36" s="28" t="inlineStr">
+      <c r="AC36" s="28" t="inlineStr">
         <is>
           <t>II.4.5</t>
         </is>
       </c>
-      <c r="Z36" s="28" t="inlineStr">
+      <c r="AD36" s="28" t="inlineStr">
         <is>
           <t>II.4.5</t>
         </is>
       </c>
-      <c r="AA36" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB36" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Dashboard dòng tiền, biểu đồ doanh thu theo ngày/tháng, phân tích tỷ trọng nguồn thu B2B và B2C.</t>
+      <c r="AE36" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF36" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Điểm vào của kế toán: doanh thu thực thu, biểu đồ 14 ngày, hàng việc cần xử lý, có số khiếu nại OPEN dẫn sang hàng chờ II.4.6. Route: /backoffice/finance</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1" s="23">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>Payment Reconciliation</t>
+          <t>Payment Complaint Queue</t>
         </is>
       </c>
       <c r="B37" s="28" t="inlineStr">
@@ -6802,7 +6970,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C37" s="28" t="n"/>
+      <c r="C37" s="29" t="n"/>
       <c r="D37" s="28" t="n"/>
       <c r="E37" s="28" t="n"/>
       <c r="F37" s="28" t="n"/>
@@ -6812,7 +6980,7 @@
       <c r="J37" s="28" t="n"/>
       <c r="K37" s="28" t="n"/>
       <c r="L37" s="28" t="n"/>
-      <c r="M37" s="28" t="n"/>
+      <c r="M37" s="29" t="n"/>
       <c r="N37" s="28" t="n"/>
       <c r="O37" s="28" t="n"/>
       <c r="P37" s="28" t="n"/>
@@ -6824,51 +6992,63 @@
       </c>
       <c r="S37" s="28" t="n"/>
       <c r="T37" s="28" t="n"/>
-      <c r="U37" s="29" t="inlineStr">
+      <c r="U37" s="28" t="n"/>
+      <c r="V37" s="28" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="W37" s="28" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="V37" s="30" t="inlineStr">
-        <is>
-          <t>UC054</t>
-        </is>
-      </c>
-      <c r="W37" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X37" s="28" t="inlineStr">
+      <c r="X37" s="28" t="n"/>
+      <c r="Y37" s="28" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="Z37" s="30" t="inlineStr">
+        <is>
+          <t>UC051</t>
+        </is>
+      </c>
+      <c r="AA37" s="31" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB37" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y37" s="28" t="inlineStr">
+      <c r="AC37" s="28" t="inlineStr">
         <is>
           <t>II.4.6</t>
         </is>
       </c>
-      <c r="Z37" s="28" t="inlineStr">
+      <c r="AD37" s="28" t="inlineStr">
         <is>
           <t>II.4.6</t>
         </is>
       </c>
-      <c r="AA37" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB37" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Đối soát dữ liệu giao dịch tự động giữa LocalPress với sao kê đối tác cổng thanh toán / ngân hàng.</t>
+      <c r="AE37" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF37" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Kế toán đối chiếu sao kê: Ghi nhận vào đơn (chạy lại hàm webhook), Cộng vào ví (TOPUP CMP-...), Từ chối bắt buộc lý do. Khóa dòng khiếu nại, xử lý lại -&gt; 409. Không có nút đánh dấu PAID. Route: /backoffice/finance/complaints</t>
         </is>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" s="23">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>Refund and Rights Management</t>
+          <t>Financial Ledger</t>
         </is>
       </c>
       <c r="B38" s="28" t="inlineStr">
@@ -6876,7 +7056,7 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C38" s="28" t="n"/>
+      <c r="C38" s="29" t="n"/>
       <c r="D38" s="28" t="n"/>
       <c r="E38" s="28" t="n"/>
       <c r="F38" s="28" t="n"/>
@@ -6884,77 +7064,65 @@
       <c r="H38" s="28" t="n"/>
       <c r="I38" s="28" t="n"/>
       <c r="J38" s="28" t="n"/>
-      <c r="K38" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="L38" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="M38" s="28" t="n"/>
+      <c r="K38" s="28" t="n"/>
+      <c r="L38" s="28" t="n"/>
+      <c r="M38" s="29" t="n"/>
       <c r="N38" s="28" t="n"/>
-      <c r="O38" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="O38" s="28" t="n"/>
       <c r="P38" s="28" t="n"/>
       <c r="Q38" s="28" t="n"/>
       <c r="R38" s="29" t="inlineStr">
         <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="S38" s="29" t="inlineStr">
-        <is>
-          <t>CRU</t>
-        </is>
-      </c>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="S38" s="28" t="n"/>
       <c r="T38" s="28" t="n"/>
       <c r="U38" s="28" t="n"/>
-      <c r="V38" s="30" t="inlineStr">
-        <is>
-          <t>UC055, UC056</t>
-        </is>
-      </c>
-      <c r="W38" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X38" s="28" t="inlineStr">
+      <c r="V38" s="28" t="n"/>
+      <c r="W38" s="28" t="n"/>
+      <c r="X38" s="28" t="n"/>
+      <c r="Y38" s="28" t="n"/>
+      <c r="Z38" s="30" t="inlineStr">
+        <is>
+          <t>UC058</t>
+        </is>
+      </c>
+      <c r="AA38" s="31" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB38" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y38" s="28" t="inlineStr">
+      <c r="AC38" s="28" t="inlineStr">
         <is>
           <t>II.4.7</t>
         </is>
       </c>
-      <c r="Z38" s="28" t="inlineStr">
+      <c r="AD38" s="28" t="inlineStr">
         <is>
           <t>II.4.7</t>
         </is>
       </c>
-      <c r="AA38" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB38" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Kiểm tra và phê duyệt yêu cầu hoàn tiền (gọi Refund API cổng thanh toán), tự động điều chỉnh quyền đọc/slot.</t>
+      <c r="AE38" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF38" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Sổ quỹ: thu (Có), hoàn (Nợ), số dư ròng; loại TOPUP khỏi doanh thu (Rule 16). Route: /backoffice/finance/ledger</t>
         </is>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1" s="23">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>Financial Reports and Alerts</t>
+          <t>Payment Orders and Financial Documents</t>
         </is>
       </c>
       <c r="B39" s="28" t="inlineStr">
@@ -6962,7 +7130,11 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C39" s="28" t="n"/>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="D39" s="28" t="n"/>
       <c r="E39" s="28" t="n"/>
       <c r="F39" s="28" t="n"/>
@@ -6972,7 +7144,7 @@
       <c r="J39" s="28" t="n"/>
       <c r="K39" s="28" t="n"/>
       <c r="L39" s="28" t="n"/>
-      <c r="M39" s="28" t="n"/>
+      <c r="M39" s="29" t="n"/>
       <c r="N39" s="28" t="n"/>
       <c r="O39" s="28" t="n"/>
       <c r="P39" s="28" t="n"/>
@@ -6982,57 +7154,53 @@
           <t>R</t>
         </is>
       </c>
-      <c r="S39" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="T39" s="29" t="inlineStr">
-        <is>
-          <t>CR</t>
-        </is>
-      </c>
+      <c r="S39" s="28" t="n"/>
+      <c r="T39" s="28" t="n"/>
       <c r="U39" s="28" t="n"/>
-      <c r="V39" s="30" t="inlineStr">
-        <is>
-          <t>UC059, UC060</t>
-        </is>
-      </c>
-      <c r="W39" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X39" s="28" t="inlineStr">
+      <c r="V39" s="28" t="n"/>
+      <c r="W39" s="28" t="n"/>
+      <c r="X39" s="28" t="n"/>
+      <c r="Y39" s="28" t="n"/>
+      <c r="Z39" s="30" t="inlineStr">
+        <is>
+          <t>UC057</t>
+        </is>
+      </c>
+      <c r="AA39" s="31" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB39" s="28" t="inlineStr">
         <is>
           <t>SV4 (Huy)</t>
         </is>
       </c>
-      <c r="Y39" s="28" t="inlineStr">
+      <c r="AC39" s="28" t="inlineStr">
         <is>
           <t>II.4.8</t>
         </is>
       </c>
-      <c r="Z39" s="28" t="inlineStr">
+      <c r="AD39" s="28" t="inlineStr">
         <is>
           <t>II.4.8</t>
         </is>
       </c>
-      <c r="AA39" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB39" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Xuất báo cáo tài chính định kỳ (Excel/PDF); hiển thị cảnh báo các khoản thanh toán treo, lỗi webhook.</t>
+      <c r="AE39" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF39" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Danh sách đơn (lọc loại, trạng thái, tìm kiếm), chi tiết các lần thanh toán, hóa đơn điện tử in / lưu PDF cho đơn đã thanh toán; nút lập đề xuất hoàn tiền dẫn sang Iter 3 (II.4.11). Route: /backoffice/finance/orders, /backoffice/finance/orders/:id</t>
         </is>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1" s="23">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>Article Editor</t>
+          <t>Payment Reconciliation</t>
         </is>
       </c>
       <c r="B40" s="28" t="inlineStr">
@@ -7040,77 +7208,73 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C40" s="28" t="n"/>
-      <c r="D40" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="28" t="n"/>
       <c r="E40" s="28" t="n"/>
-      <c r="F40" s="29" t="inlineStr">
-        <is>
-          <t>CR</t>
-        </is>
-      </c>
-      <c r="G40" s="29" t="inlineStr">
-        <is>
-          <t>CR</t>
-        </is>
-      </c>
+      <c r="F40" s="28" t="n"/>
+      <c r="G40" s="28" t="n"/>
       <c r="H40" s="28" t="n"/>
       <c r="I40" s="28" t="n"/>
       <c r="J40" s="28" t="n"/>
       <c r="K40" s="28" t="n"/>
       <c r="L40" s="28" t="n"/>
-      <c r="M40" s="28" t="n"/>
+      <c r="M40" s="29" t="n"/>
       <c r="N40" s="28" t="n"/>
       <c r="O40" s="28" t="n"/>
       <c r="P40" s="28" t="n"/>
       <c r="Q40" s="28" t="n"/>
-      <c r="R40" s="28" t="n"/>
+      <c r="R40" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="S40" s="28" t="n"/>
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
-      <c r="V40" s="30" t="inlineStr">
-        <is>
-          <t>UC061</t>
-        </is>
-      </c>
-      <c r="W40" s="31" t="inlineStr">
-        <is>
-          <t>Iter 1</t>
-        </is>
-      </c>
-      <c r="X40" s="28" t="inlineStr">
-        <is>
-          <t>SV5 (Tùng)</t>
-        </is>
-      </c>
-      <c r="Y40" s="28" t="inlineStr">
-        <is>
-          <t>II.5.1</t>
-        </is>
-      </c>
-      <c r="Z40" s="28" t="inlineStr">
-        <is>
-          <t>II.5.1</t>
-        </is>
-      </c>
-      <c r="AA40" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB40" s="30" t="inlineStr">
-        <is>
-          <t>[Đầu quy trình] Trình soạn thảo bài viết phong phú (WYSIWYG/Markdown), nhập tiêu đề, sapo, nội dung bài draft, tác giả.</t>
+      <c r="V40" s="28" t="n"/>
+      <c r="W40" s="28" t="n"/>
+      <c r="X40" s="28" t="n"/>
+      <c r="Y40" s="28" t="n"/>
+      <c r="Z40" s="30" t="inlineStr">
+        <is>
+          <t>UC054</t>
+        </is>
+      </c>
+      <c r="AA40" s="31" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB40" s="28" t="inlineStr">
+        <is>
+          <t>SV4 (Huy)</t>
+        </is>
+      </c>
+      <c r="AC40" s="28" t="inlineStr">
+        <is>
+          <t>II.4.9</t>
+        </is>
+      </c>
+      <c r="AD40" s="28" t="inlineStr">
+        <is>
+          <t>II.4.9</t>
+        </is>
+      </c>
+      <c r="AE40" s="28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AF40" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Đối soát kỳ, xử lý khoản lệch, kế toán trưởng chốt kỳ. Sao kê đang giả lập bằng tổng hệ thống, khoản lệch lưu trong bộ nhớ. Route: /backoffice/finance/reconciliation</t>
         </is>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1" s="23">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>Article Metadata and Media</t>
+          <t>Advertiser Receivables</t>
         </is>
       </c>
       <c r="B41" s="28" t="inlineStr">
@@ -7118,77 +7282,81 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C41" s="28" t="n"/>
-      <c r="D41" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="C41" s="29" t="n"/>
+      <c r="D41" s="28" t="n"/>
       <c r="E41" s="28" t="n"/>
-      <c r="F41" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="G41" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="F41" s="28" t="n"/>
+      <c r="G41" s="28" t="n"/>
       <c r="H41" s="28" t="n"/>
       <c r="I41" s="28" t="n"/>
       <c r="J41" s="28" t="n"/>
       <c r="K41" s="28" t="n"/>
       <c r="L41" s="28" t="n"/>
-      <c r="M41" s="28" t="n"/>
+      <c r="M41" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="N41" s="28" t="n"/>
-      <c r="O41" s="28" t="n"/>
+      <c r="O41" s="28" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="P41" s="28" t="n"/>
       <c r="Q41" s="28" t="n"/>
-      <c r="R41" s="28" t="n"/>
+      <c r="R41" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="S41" s="28" t="n"/>
       <c r="T41" s="28" t="n"/>
       <c r="U41" s="28" t="n"/>
-      <c r="V41" s="30" t="inlineStr">
-        <is>
-          <t>UC063, UC064</t>
-        </is>
-      </c>
-      <c r="W41" s="31" t="inlineStr">
-        <is>
-          <t>Iter 1</t>
-        </is>
-      </c>
-      <c r="X41" s="28" t="inlineStr">
-        <is>
-          <t>SV5 (Tùng)</t>
-        </is>
-      </c>
-      <c r="Y41" s="28" t="inlineStr">
-        <is>
-          <t>II.5.2</t>
-        </is>
-      </c>
-      <c r="Z41" s="28" t="inlineStr">
-        <is>
-          <t>II.5.2</t>
-        </is>
-      </c>
-      <c r="AA41" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB41" s="30" t="inlineStr">
-        <is>
-          <t>[Đầu quy trình] Quản lý danh mục, tag, thông tin địa phương cấp tỉnh, slug URL, tải lên thumbnail và quản lý media.</t>
+      <c r="V41" s="28" t="n"/>
+      <c r="W41" s="28" t="n"/>
+      <c r="X41" s="28" t="n"/>
+      <c r="Y41" s="28" t="n"/>
+      <c r="Z41" s="30" t="inlineStr">
+        <is>
+          <t>UC053</t>
+        </is>
+      </c>
+      <c r="AA41" s="31" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB41" s="28" t="inlineStr">
+        <is>
+          <t>SV4 (Huy)</t>
+        </is>
+      </c>
+      <c r="AC41" s="28" t="inlineStr">
+        <is>
+          <t>II.4.10</t>
+        </is>
+      </c>
+      <c r="AD41" s="28" t="inlineStr">
+        <is>
+          <t>II.4.10</t>
+        </is>
+      </c>
+      <c r="AE41" s="28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AF41" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Công nợ quảng cáo theo chiến dịch. Đã có API GET /finance/receivables, chưa có màn hình, chưa có nhắc nợ. Route: (chưa có)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="24" customHeight="1" s="23">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>Article Version History</t>
+          <t>Refund and Rights Management</t>
         </is>
       </c>
       <c r="B42" s="28" t="inlineStr">
@@ -7196,73 +7364,85 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C42" s="28" t="n"/>
+      <c r="C42" s="29" t="n"/>
       <c r="D42" s="28" t="n"/>
       <c r="E42" s="28" t="n"/>
-      <c r="F42" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G42" s="29" t="inlineStr">
-        <is>
-          <t>CRU</t>
-        </is>
-      </c>
+      <c r="F42" s="28" t="n"/>
+      <c r="G42" s="28" t="n"/>
       <c r="H42" s="28" t="n"/>
       <c r="I42" s="28" t="n"/>
       <c r="J42" s="28" t="n"/>
       <c r="K42" s="28" t="n"/>
       <c r="L42" s="28" t="n"/>
-      <c r="M42" s="28" t="n"/>
+      <c r="M42" s="29" t="n"/>
       <c r="N42" s="28" t="n"/>
       <c r="O42" s="28" t="n"/>
       <c r="P42" s="28" t="n"/>
       <c r="Q42" s="28" t="n"/>
-      <c r="R42" s="28" t="n"/>
-      <c r="S42" s="28" t="n"/>
+      <c r="R42" s="29" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
+      <c r="S42" s="28" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
-      <c r="V42" s="30" t="inlineStr">
-        <is>
-          <t>UC062</t>
-        </is>
-      </c>
-      <c r="W42" s="32" t="inlineStr">
-        <is>
-          <t>Iter 2</t>
-        </is>
-      </c>
-      <c r="X42" s="28" t="inlineStr">
-        <is>
-          <t>SV5 (Tùng)</t>
-        </is>
-      </c>
-      <c r="Y42" s="28" t="inlineStr">
-        <is>
-          <t>II.5.3</t>
-        </is>
-      </c>
-      <c r="Z42" s="28" t="inlineStr">
-        <is>
-          <t>II.5.3</t>
-        </is>
-      </c>
-      <c r="AA42" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB42" s="30" t="inlineStr">
-        <is>
-          <t>[Giữa quy trình] Quản lý lịch sử các phiên bản bài viết; giao diện so sánh khác biệt nội dung (diff) và khôi phục bản cũ.</t>
+      <c r="V42" s="28" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="W42" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X42" s="28" t="n"/>
+      <c r="Y42" s="28" t="n"/>
+      <c r="Z42" s="30" t="inlineStr">
+        <is>
+          <t>UC055, UC056</t>
+        </is>
+      </c>
+      <c r="AA42" s="31" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB42" s="28" t="inlineStr">
+        <is>
+          <t>SV4 (Huy)</t>
+        </is>
+      </c>
+      <c r="AC42" s="28" t="inlineStr">
+        <is>
+          <t>II.4.11</t>
+        </is>
+      </c>
+      <c r="AD42" s="28" t="inlineStr">
+        <is>
+          <t>II.4.11</t>
+        </is>
+      </c>
+      <c r="AE42" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="AF42" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Hoàn tiền 4 mắt, Refund Cap, giao dịch REFUND, hoàn vào ví cho đơn trả bằng ví, phát RefundCompletedEvent. Listener thu hồi quyền của SV1 / SV3 chưa có. Route: /backoffice/finance/refunds</t>
         </is>
       </c>
     </row>
     <row r="43" ht="24" customHeight="1" s="23">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>Article Submission and Revision</t>
+          <t>Financial Reports and Alerts</t>
         </is>
       </c>
       <c r="B43" s="28" t="inlineStr">
@@ -7270,77 +7450,81 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C43" s="28" t="n"/>
+      <c r="C43" s="29" t="n"/>
       <c r="D43" s="28" t="n"/>
       <c r="E43" s="28" t="n"/>
-      <c r="F43" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="G43" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="F43" s="28" t="n"/>
+      <c r="G43" s="28" t="n"/>
       <c r="H43" s="28" t="n"/>
       <c r="I43" s="28" t="n"/>
       <c r="J43" s="28" t="n"/>
       <c r="K43" s="28" t="n"/>
       <c r="L43" s="28" t="n"/>
-      <c r="M43" s="28" t="n"/>
+      <c r="M43" s="29" t="n"/>
       <c r="N43" s="28" t="n"/>
       <c r="O43" s="28" t="n"/>
       <c r="P43" s="28" t="n"/>
       <c r="Q43" s="28" t="n"/>
-      <c r="R43" s="28" t="n"/>
-      <c r="S43" s="28" t="n"/>
-      <c r="T43" s="29" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="R43" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="S43" s="28" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
-      <c r="V43" s="30" t="inlineStr">
-        <is>
-          <t>UC066, UC067</t>
-        </is>
-      </c>
-      <c r="W43" s="32" t="inlineStr">
-        <is>
-          <t>Iter 2</t>
-        </is>
-      </c>
-      <c r="X43" s="28" t="inlineStr">
-        <is>
-          <t>SV5 (Tùng)</t>
-        </is>
-      </c>
+      <c r="V43" s="28" t="n"/>
+      <c r="W43" s="28" t="n"/>
+      <c r="X43" s="28" t="n"/>
       <c r="Y43" s="28" t="inlineStr">
         <is>
-          <t>II.5.4</t>
-        </is>
-      </c>
-      <c r="Z43" s="28" t="inlineStr">
-        <is>
-          <t>II.5.4</t>
-        </is>
-      </c>
-      <c r="AA43" s="28" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="AB43" s="30" t="inlineStr">
-        <is>
-          <t>[Giữa quy trình] Xem trước bài viết (preview), nộp bài draft lên hàng đợi duyệt của SV2; nhận thông báo phản hồi và gửi lại bản sửa.</t>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Z43" s="30" t="inlineStr">
+        <is>
+          <t>UC060, UC059</t>
+        </is>
+      </c>
+      <c r="AA43" s="31" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB43" s="28" t="inlineStr">
+        <is>
+          <t>SV4 (Huy)</t>
+        </is>
+      </c>
+      <c r="AC43" s="28" t="inlineStr">
+        <is>
+          <t>II.4.12</t>
+        </is>
+      </c>
+      <c r="AD43" s="28" t="inlineStr">
+        <is>
+          <t>II.4.12</t>
+        </is>
+      </c>
+      <c r="AE43" s="28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AF43" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Cảnh báo (REFUND_PENDING, COMPLAINT_OPEN, DEBT_OVERDUE) và xuất CSV. Đã có API, chưa có màn hình, CSV chưa lọc theo ngày. Route: (chưa có)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="24" customHeight="1" s="23">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>Content Access and Paywall</t>
+          <t>Article Editor</t>
         </is>
       </c>
       <c r="B44" s="28" t="inlineStr">
@@ -7349,27 +7533,27 @@
         </is>
       </c>
       <c r="C44" s="28" t="n"/>
-      <c r="D44" s="28" t="n"/>
+      <c r="D44" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="E44" s="28" t="n"/>
       <c r="F44" s="29" t="inlineStr">
         <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n"/>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="G44" s="29" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
       <c r="H44" s="28" t="n"/>
       <c r="I44" s="28" t="n"/>
       <c r="J44" s="28" t="n"/>
-      <c r="K44" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="L44" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="K44" s="28" t="n"/>
+      <c r="L44" s="28" t="n"/>
       <c r="M44" s="28" t="n"/>
       <c r="N44" s="28" t="n"/>
       <c r="O44" s="28" t="n"/>
@@ -7379,46 +7563,50 @@
       <c r="S44" s="28" t="n"/>
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
-      <c r="V44" s="30" t="inlineStr">
-        <is>
-          <t>UC068, UC069</t>
-        </is>
-      </c>
-      <c r="W44" s="32" t="inlineStr">
-        <is>
-          <t>Iter 2</t>
-        </is>
-      </c>
-      <c r="X44" s="28" t="inlineStr">
+      <c r="V44" s="28" t="n"/>
+      <c r="W44" s="28" t="n"/>
+      <c r="X44" s="28" t="n"/>
+      <c r="Y44" s="28" t="n"/>
+      <c r="Z44" s="30" t="inlineStr">
+        <is>
+          <t>UC061</t>
+        </is>
+      </c>
+      <c r="AA44" s="31" t="inlineStr">
+        <is>
+          <t>Iter 1</t>
+        </is>
+      </c>
+      <c r="AB44" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y44" s="28" t="inlineStr">
-        <is>
-          <t>II.5.5</t>
-        </is>
-      </c>
-      <c r="Z44" s="28" t="inlineStr">
-        <is>
-          <t>II.5.5</t>
-        </is>
-      </c>
-      <c r="AA44" s="28" t="inlineStr">
+      <c r="AC44" s="28" t="inlineStr">
+        <is>
+          <t>II.5.1</t>
+        </is>
+      </c>
+      <c r="AD44" s="28" t="inlineStr">
+        <is>
+          <t>II.5.1</t>
+        </is>
+      </c>
+      <c r="AE44" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB44" s="30" t="inlineStr">
-        <is>
-          <t>[Giữa quy trình] Cấu hình chính sách truy cập (Free / Premium / Mua lẻ); Back-end PaywallEngine kiểm tra quyền ở server-side.</t>
+      <c r="AF44" s="30" t="inlineStr">
+        <is>
+          <t>[Đầu quy trình] Trình soạn thảo bài viết phong phú (WYSIWYG/Markdown), nhập tiêu đề, sapo, nội dung bài draft, tác giả.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="24" customHeight="1" s="23">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>AI Editorial Assistant</t>
+          <t>Article Metadata and Media</t>
         </is>
       </c>
       <c r="B45" s="28" t="inlineStr">
@@ -7427,9 +7615,17 @@
         </is>
       </c>
       <c r="C45" s="28" t="n"/>
-      <c r="D45" s="28" t="n"/>
+      <c r="D45" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="E45" s="28" t="n"/>
-      <c r="F45" s="28" t="n"/>
+      <c r="F45" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="G45" s="29" t="inlineStr">
         <is>
           <t>RU</t>
@@ -7448,51 +7644,51 @@
       <c r="R45" s="28" t="n"/>
       <c r="S45" s="28" t="n"/>
       <c r="T45" s="28" t="n"/>
-      <c r="U45" s="29" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V45" s="30" t="inlineStr">
-        <is>
-          <t>UC065</t>
-        </is>
-      </c>
-      <c r="W45" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X45" s="28" t="inlineStr">
+      <c r="U45" s="28" t="n"/>
+      <c r="V45" s="28" t="n"/>
+      <c r="W45" s="28" t="n"/>
+      <c r="X45" s="28" t="n"/>
+      <c r="Y45" s="28" t="n"/>
+      <c r="Z45" s="30" t="inlineStr">
+        <is>
+          <t>UC063, UC064</t>
+        </is>
+      </c>
+      <c r="AA45" s="31" t="inlineStr">
+        <is>
+          <t>Iter 1</t>
+        </is>
+      </c>
+      <c r="AB45" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y45" s="28" t="inlineStr">
-        <is>
-          <t>II.5.6</t>
-        </is>
-      </c>
-      <c r="Z45" s="28" t="inlineStr">
-        <is>
-          <t>II.5.6</t>
-        </is>
-      </c>
-      <c r="AA45" s="28" t="inlineStr">
+      <c r="AC45" s="28" t="inlineStr">
+        <is>
+          <t>II.5.2</t>
+        </is>
+      </c>
+      <c r="AD45" s="28" t="inlineStr">
+        <is>
+          <t>II.5.2</t>
+        </is>
+      </c>
+      <c r="AE45" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB45" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Gọi API AI (Gemini/OpenAI) gợi ý tiêu đề chuẩn SEO, tự động tóm tắt sapo, gợi ý bộ thẻ tag và sinh alt text.</t>
+      <c r="AF45" s="30" t="inlineStr">
+        <is>
+          <t>[Đầu quy trình] Quản lý danh mục, tag, thông tin địa phương cấp tỉnh, slug URL, tải lên thumbnail và quản lý media.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1" s="23">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>Advertising Slot Configuration</t>
+          <t>Article Version History</t>
         </is>
       </c>
       <c r="B46" s="28" t="inlineStr">
@@ -7503,19 +7699,23 @@
       <c r="C46" s="28" t="n"/>
       <c r="D46" s="28" t="n"/>
       <c r="E46" s="28" t="n"/>
-      <c r="F46" s="28" t="n"/>
-      <c r="G46" s="28" t="n"/>
+      <c r="F46" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G46" s="29" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
       <c r="H46" s="28" t="n"/>
       <c r="I46" s="28" t="n"/>
       <c r="J46" s="28" t="n"/>
       <c r="K46" s="28" t="n"/>
       <c r="L46" s="28" t="n"/>
       <c r="M46" s="28" t="n"/>
-      <c r="N46" s="29" t="inlineStr">
-        <is>
-          <t>CRUD</t>
-        </is>
-      </c>
+      <c r="N46" s="28" t="n"/>
       <c r="O46" s="28" t="n"/>
       <c r="P46" s="28" t="n"/>
       <c r="Q46" s="28" t="n"/>
@@ -7523,46 +7723,50 @@
       <c r="S46" s="28" t="n"/>
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
-      <c r="V46" s="30" t="inlineStr">
-        <is>
-          <t>UC070</t>
-        </is>
-      </c>
-      <c r="W46" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X46" s="28" t="inlineStr">
+      <c r="V46" s="28" t="n"/>
+      <c r="W46" s="28" t="n"/>
+      <c r="X46" s="28" t="n"/>
+      <c r="Y46" s="28" t="n"/>
+      <c r="Z46" s="30" t="inlineStr">
+        <is>
+          <t>UC062</t>
+        </is>
+      </c>
+      <c r="AA46" s="32" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB46" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y46" s="28" t="inlineStr">
-        <is>
-          <t>II.5.7</t>
-        </is>
-      </c>
-      <c r="Z46" s="28" t="inlineStr">
-        <is>
-          <t>II.5.7</t>
-        </is>
-      </c>
-      <c r="AA46" s="28" t="inlineStr">
+      <c r="AC46" s="28" t="inlineStr">
+        <is>
+          <t>II.5.3</t>
+        </is>
+      </c>
+      <c r="AD46" s="28" t="inlineStr">
+        <is>
+          <t>II.5.3</t>
+        </is>
+      </c>
+      <c r="AE46" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB46" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Admin cấu hình vị trí đặt banner trên layout (header, sidebar, in-article), kích thước chuẩn, định giá gốc.</t>
+      <c r="AF46" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Quản lý lịch sử các phiên bản bài viết; giao diện so sánh khác biệt nội dung (diff) và khôi phục bản cũ.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="24" customHeight="1" s="23">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>Advertisement Delivery and Tracking</t>
+          <t>Article Submission and Revision</t>
         </is>
       </c>
       <c r="B47" s="28" t="inlineStr">
@@ -7573,78 +7777,78 @@
       <c r="C47" s="28" t="n"/>
       <c r="D47" s="28" t="n"/>
       <c r="E47" s="28" t="n"/>
-      <c r="F47" s="28" t="n"/>
-      <c r="G47" s="28" t="n"/>
+      <c r="F47" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="G47" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="H47" s="28" t="n"/>
       <c r="I47" s="28" t="n"/>
       <c r="J47" s="28" t="n"/>
       <c r="K47" s="28" t="n"/>
       <c r="L47" s="28" t="n"/>
       <c r="M47" s="28" t="n"/>
-      <c r="N47" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="O47" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="P47" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="Q47" s="29" t="inlineStr">
-        <is>
-          <t>CRU</t>
-        </is>
-      </c>
+      <c r="N47" s="28" t="n"/>
+      <c r="O47" s="28" t="n"/>
+      <c r="P47" s="28" t="n"/>
+      <c r="Q47" s="28" t="n"/>
       <c r="R47" s="28" t="n"/>
       <c r="S47" s="28" t="n"/>
-      <c r="T47" s="28" t="n"/>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="U47" s="28" t="n"/>
-      <c r="V47" s="30" t="inlineStr">
-        <is>
-          <t>UC071, UC072</t>
-        </is>
-      </c>
-      <c r="W47" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X47" s="28" t="inlineStr">
+      <c r="V47" s="28" t="n"/>
+      <c r="W47" s="28" t="n"/>
+      <c r="X47" s="28" t="n"/>
+      <c r="Y47" s="28" t="n"/>
+      <c r="Z47" s="30" t="inlineStr">
+        <is>
+          <t>UC066, UC067</t>
+        </is>
+      </c>
+      <c r="AA47" s="32" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB47" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y47" s="28" t="inlineStr">
-        <is>
-          <t>II.5.8</t>
-        </is>
-      </c>
-      <c r="Z47" s="28" t="inlineStr">
-        <is>
-          <t>II.5.8</t>
-        </is>
-      </c>
-      <c r="AA47" s="28" t="inlineStr">
+      <c r="AC47" s="28" t="inlineStr">
+        <is>
+          <t>II.5.4</t>
+        </is>
+      </c>
+      <c r="AD47" s="28" t="inlineStr">
+        <is>
+          <t>II.5.4</t>
+        </is>
+      </c>
+      <c r="AE47" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB47" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Engine phân phối banner hợp lệ theo slot và thời gian thực; ghi nhận sự kiện Impression và Click chống gian lận.</t>
+      <c r="AF47" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Xem trước bài viết (preview), nộp bài draft lên hàng đợi duyệt của SV2; nhận thông báo phản hồi và gửi lại bản sửa.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="24" customHeight="1" s="23">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>Advertisement URL Monitoring</t>
+          <t>Content Access and Paywall</t>
         </is>
       </c>
       <c r="B48" s="28" t="inlineStr">
@@ -7655,70 +7859,78 @@
       <c r="C48" s="28" t="n"/>
       <c r="D48" s="28" t="n"/>
       <c r="E48" s="28" t="n"/>
-      <c r="F48" s="28" t="n"/>
+      <c r="F48" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="G48" s="28" t="n"/>
       <c r="H48" s="28" t="n"/>
       <c r="I48" s="28" t="n"/>
       <c r="J48" s="28" t="n"/>
-      <c r="K48" s="28" t="n"/>
-      <c r="L48" s="28" t="n"/>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="M48" s="28" t="n"/>
       <c r="N48" s="28" t="n"/>
       <c r="O48" s="28" t="n"/>
-      <c r="P48" s="29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
+      <c r="P48" s="28" t="n"/>
       <c r="Q48" s="28" t="n"/>
       <c r="R48" s="28" t="n"/>
       <c r="S48" s="28" t="n"/>
       <c r="T48" s="28" t="n"/>
-      <c r="U48" s="29" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V48" s="30" t="inlineStr">
-        <is>
-          <t>UC073</t>
-        </is>
-      </c>
-      <c r="W48" s="33" t="inlineStr">
-        <is>
-          <t>Iter 3</t>
-        </is>
-      </c>
-      <c r="X48" s="28" t="inlineStr">
+      <c r="U48" s="28" t="n"/>
+      <c r="V48" s="28" t="n"/>
+      <c r="W48" s="28" t="n"/>
+      <c r="X48" s="28" t="n"/>
+      <c r="Y48" s="28" t="n"/>
+      <c r="Z48" s="30" t="inlineStr">
+        <is>
+          <t>UC068, UC069</t>
+        </is>
+      </c>
+      <c r="AA48" s="32" t="inlineStr">
+        <is>
+          <t>Iter 2</t>
+        </is>
+      </c>
+      <c r="AB48" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y48" s="28" t="inlineStr">
-        <is>
-          <t>II.5.9</t>
-        </is>
-      </c>
-      <c r="Z48" s="28" t="inlineStr">
-        <is>
-          <t>II.5.9</t>
-        </is>
-      </c>
-      <c r="AA48" s="28" t="inlineStr">
+      <c r="AC48" s="28" t="inlineStr">
+        <is>
+          <t>II.5.5</t>
+        </is>
+      </c>
+      <c r="AD48" s="28" t="inlineStr">
+        <is>
+          <t>II.5.5</t>
+        </is>
+      </c>
+      <c r="AE48" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB48" s="30" t="inlineStr">
-        <is>
-          <t>[Cuối quy trình] Tác vụ nền (Background Job) định kỳ kiểm tra sức khỏe URL đích của quảng cáo (phát hiện liên kết chết, redirect độc hại).</t>
+      <c r="AF48" s="30" t="inlineStr">
+        <is>
+          <t>[Giữa quy trình] Cấu hình chính sách truy cập (Free / Premium / Mua lẻ); Back-end PaywallEngine kiểm tra quyền ở server-side.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1" s="23">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>System Administration Console</t>
+          <t>AI Editorial Assistant</t>
         </is>
       </c>
       <c r="B49" s="28" t="inlineStr">
@@ -7726,15 +7938,15 @@
           <t>Screen</t>
         </is>
       </c>
-      <c r="C49" s="29" t="inlineStr">
-        <is>
-          <t>CRUD</t>
-        </is>
-      </c>
+      <c r="C49" s="28" t="n"/>
       <c r="D49" s="28" t="n"/>
       <c r="E49" s="28" t="n"/>
       <c r="F49" s="28" t="n"/>
-      <c r="G49" s="28" t="n"/>
+      <c r="G49" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="H49" s="28" t="n"/>
       <c r="I49" s="28" t="n"/>
       <c r="J49" s="28" t="n"/>
@@ -7747,47 +7959,367 @@
       <c r="Q49" s="28" t="n"/>
       <c r="R49" s="28" t="n"/>
       <c r="S49" s="28" t="n"/>
-      <c r="T49" s="29" t="inlineStr">
+      <c r="T49" s="28" t="n"/>
+      <c r="U49" s="29" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="U49" s="29" t="inlineStr">
+      <c r="V49" s="29" t="n"/>
+      <c r="W49" s="29" t="n"/>
+      <c r="X49" s="29" t="n"/>
+      <c r="Y49" s="29" t="n"/>
+      <c r="Z49" s="30" t="inlineStr">
+        <is>
+          <t>UC065</t>
+        </is>
+      </c>
+      <c r="AA49" s="33" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB49" s="28" t="inlineStr">
+        <is>
+          <t>SV5 (Tùng)</t>
+        </is>
+      </c>
+      <c r="AC49" s="28" t="inlineStr">
+        <is>
+          <t>II.5.6</t>
+        </is>
+      </c>
+      <c r="AD49" s="28" t="inlineStr">
+        <is>
+          <t>II.5.6</t>
+        </is>
+      </c>
+      <c r="AE49" s="28" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AF49" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Gọi API AI (Gemini/OpenAI) gợi ý tiêu đề chuẩn SEO, tự động tóm tắt sapo, gợi ý bộ thẻ tag và sinh alt text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1" s="23">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>Advertising Slot Configuration</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C50" s="28" t="n"/>
+      <c r="D50" s="28" t="n"/>
+      <c r="E50" s="28" t="n"/>
+      <c r="F50" s="28" t="n"/>
+      <c r="G50" s="28" t="n"/>
+      <c r="H50" s="28" t="n"/>
+      <c r="I50" s="28" t="n"/>
+      <c r="J50" s="28" t="n"/>
+      <c r="K50" s="28" t="n"/>
+      <c r="L50" s="28" t="n"/>
+      <c r="M50" s="28" t="n"/>
+      <c r="N50" s="29" t="inlineStr">
+        <is>
+          <t>CRUD</t>
+        </is>
+      </c>
+      <c r="O50" s="28" t="n"/>
+      <c r="P50" s="28" t="n"/>
+      <c r="Q50" s="28" t="n"/>
+      <c r="R50" s="28" t="n"/>
+      <c r="S50" s="28" t="n"/>
+      <c r="T50" s="28" t="n"/>
+      <c r="U50" s="28" t="n"/>
+      <c r="V50" s="28" t="n"/>
+      <c r="W50" s="28" t="n"/>
+      <c r="X50" s="28" t="n"/>
+      <c r="Y50" s="28" t="n"/>
+      <c r="Z50" s="30" t="inlineStr">
+        <is>
+          <t>UC070</t>
+        </is>
+      </c>
+      <c r="AA50" s="33" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB50" s="28" t="inlineStr">
+        <is>
+          <t>SV5 (Tùng)</t>
+        </is>
+      </c>
+      <c r="AC50" s="28" t="inlineStr">
+        <is>
+          <t>II.5.7</t>
+        </is>
+      </c>
+      <c r="AD50" s="28" t="inlineStr">
+        <is>
+          <t>II.5.7</t>
+        </is>
+      </c>
+      <c r="AE50" s="28" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AF50" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Admin cấu hình vị trí đặt banner trên layout (header, sidebar, in-article), kích thước chuẩn, định giá gốc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1" s="23">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>Advertisement Delivery and Tracking</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="n"/>
+      <c r="D51" s="28" t="n"/>
+      <c r="E51" s="28" t="n"/>
+      <c r="F51" s="28" t="n"/>
+      <c r="G51" s="28" t="n"/>
+      <c r="H51" s="28" t="n"/>
+      <c r="I51" s="28" t="n"/>
+      <c r="J51" s="28" t="n"/>
+      <c r="K51" s="28" t="n"/>
+      <c r="L51" s="28" t="n"/>
+      <c r="M51" s="28" t="n"/>
+      <c r="N51" s="29" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="V49" s="30" t="inlineStr">
+      <c r="O51" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="P51" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Q51" s="29" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
+      <c r="R51" s="28" t="n"/>
+      <c r="S51" s="28" t="n"/>
+      <c r="T51" s="28" t="n"/>
+      <c r="U51" s="28" t="n"/>
+      <c r="V51" s="28" t="n"/>
+      <c r="W51" s="28" t="n"/>
+      <c r="X51" s="28" t="n"/>
+      <c r="Y51" s="28" t="n"/>
+      <c r="Z51" s="30" t="inlineStr">
+        <is>
+          <t>UC071, UC072</t>
+        </is>
+      </c>
+      <c r="AA51" s="33" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB51" s="28" t="inlineStr">
+        <is>
+          <t>SV5 (Tùng)</t>
+        </is>
+      </c>
+      <c r="AC51" s="28" t="inlineStr">
+        <is>
+          <t>II.5.8</t>
+        </is>
+      </c>
+      <c r="AD51" s="28" t="inlineStr">
+        <is>
+          <t>II.5.8</t>
+        </is>
+      </c>
+      <c r="AE51" s="28" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AF51" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Engine phân phối banner hợp lệ theo slot và thời gian thực; ghi nhận sự kiện Impression và Click chống gian lận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1" s="23">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>Advertisement URL Monitoring</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="n"/>
+      <c r="D52" s="28" t="n"/>
+      <c r="E52" s="28" t="n"/>
+      <c r="F52" s="28" t="n"/>
+      <c r="G52" s="28" t="n"/>
+      <c r="H52" s="28" t="n"/>
+      <c r="I52" s="28" t="n"/>
+      <c r="J52" s="28" t="n"/>
+      <c r="K52" s="28" t="n"/>
+      <c r="L52" s="28" t="n"/>
+      <c r="M52" s="28" t="n"/>
+      <c r="N52" s="28" t="n"/>
+      <c r="O52" s="28" t="n"/>
+      <c r="P52" s="29" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="Q52" s="28" t="n"/>
+      <c r="R52" s="28" t="n"/>
+      <c r="S52" s="28" t="n"/>
+      <c r="T52" s="28" t="n"/>
+      <c r="U52" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V52" s="29" t="n"/>
+      <c r="W52" s="29" t="n"/>
+      <c r="X52" s="29" t="n"/>
+      <c r="Y52" s="29" t="n"/>
+      <c r="Z52" s="30" t="inlineStr">
+        <is>
+          <t>UC073</t>
+        </is>
+      </c>
+      <c r="AA52" s="33" t="inlineStr">
+        <is>
+          <t>Iter 3</t>
+        </is>
+      </c>
+      <c r="AB52" s="28" t="inlineStr">
+        <is>
+          <t>SV5 (Tùng)</t>
+        </is>
+      </c>
+      <c r="AC52" s="28" t="inlineStr">
+        <is>
+          <t>II.5.9</t>
+        </is>
+      </c>
+      <c r="AD52" s="28" t="inlineStr">
+        <is>
+          <t>II.5.9</t>
+        </is>
+      </c>
+      <c r="AE52" s="28" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="AF52" s="30" t="inlineStr">
+        <is>
+          <t>[Cuối quy trình] Tác vụ nền (Background Job) định kỳ kiểm tra sức khỏe URL đích của quảng cáo (phát hiện liên kết chết, redirect độc hại).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1" s="23">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>System Administration Console</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>CRUD</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="n"/>
+      <c r="E53" s="28" t="n"/>
+      <c r="F53" s="28" t="n"/>
+      <c r="G53" s="28" t="n"/>
+      <c r="H53" s="28" t="n"/>
+      <c r="I53" s="28" t="n"/>
+      <c r="J53" s="28" t="n"/>
+      <c r="K53" s="28" t="n"/>
+      <c r="L53" s="28" t="n"/>
+      <c r="M53" s="28" t="n"/>
+      <c r="N53" s="28" t="n"/>
+      <c r="O53" s="28" t="n"/>
+      <c r="P53" s="28" t="n"/>
+      <c r="Q53" s="28" t="n"/>
+      <c r="R53" s="28" t="n"/>
+      <c r="S53" s="28" t="n"/>
+      <c r="T53" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U53" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="V53" s="29" t="n"/>
+      <c r="W53" s="29" t="n"/>
+      <c r="X53" s="29" t="n"/>
+      <c r="Y53" s="29" t="n"/>
+      <c r="Z53" s="30" t="inlineStr">
         <is>
           <t>UC074, UC075, UC076, UC077</t>
         </is>
       </c>
-      <c r="W49" s="33" t="inlineStr">
+      <c r="AA53" s="33" t="inlineStr">
         <is>
           <t>Iter 3</t>
         </is>
       </c>
-      <c r="X49" s="28" t="inlineStr">
+      <c r="AB53" s="28" t="inlineStr">
         <is>
           <t>SV5 (Tùng)</t>
         </is>
       </c>
-      <c r="Y49" s="28" t="inlineStr">
+      <c r="AC53" s="28" t="inlineStr">
         <is>
           <t>II.5.10</t>
         </is>
       </c>
-      <c r="Z49" s="28" t="inlineStr">
+      <c r="AD53" s="28" t="inlineStr">
         <is>
           <t>II.5.10</t>
         </is>
       </c>
-      <c r="AA49" s="28" t="inlineStr">
+      <c r="AE53" s="28" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="AB49" s="30" t="inlineStr">
+      <c r="AF53" s="30" t="inlineStr">
         <is>
           <t>[Cuối quy trình] Quản trị tài khoản, vai trò và phân quyền (RBAC); tra cứu nhật ký audit log; giám sát background job và sao lưu DB.</t>
         </is>

</xml_diff>